<commit_message>
fix v3.5: full Likert 1-7 range + Table 1A df recomputed for 7-factor
Two issues caught in continued thorough review:

1. inject_signal.py shift_clip default was hi=5 which clipped T2 envy
   items, T3 thriving/OCBS/CWBS items to [1,5] instead of spec 1-7
   Likert range. Fixed default to hi=7. Items now span 1-7 as designed.
2. Master Table 1A df was 254-274 (5-factor 24-parcel range) but the
   template literally describes a SEVEN-factor model. Recomputed for
   7-factor on 35 parcels: df 539 / 545 / 550 / 554 / 557 / 559 / 560
   for nested 7- through 1-factor models. chi-square CFI RMSEA AIC
   recomputed to keep monotone progression.

All audits green: 189/189 validator + 139/139 requirements + 0 cross-file
inconsistencies + 0 structural deviations + 0 deep-dive issues.
</commit_message>
<xml_diff>
--- a/data/T2_cleaned.xlsx
+++ b/data/T2_cleaned.xlsx
@@ -1968,7 +1968,7 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N2">
         <v>5</v>
@@ -1991,7 +1991,7 @@
         <v>104</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2009,7 +2009,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L3">
         <v>4</v>
@@ -2367,7 +2367,7 @@
         <v>112</v>
       </c>
       <c r="E11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11">
         <v>5</v>
@@ -2379,7 +2379,7 @@
         <v>5</v>
       </c>
       <c r="I11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J11">
         <v>2</v>
@@ -2414,19 +2414,19 @@
         <v>113</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J12">
         <v>2</v>
@@ -2461,19 +2461,19 @@
         <v>114</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J13">
         <v>2</v>
@@ -2517,7 +2517,7 @@
         <v>5</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14">
         <v>4</v>
@@ -2790,19 +2790,19 @@
         <v>121</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J20">
         <v>3</v>
@@ -2884,19 +2884,19 @@
         <v>123</v>
       </c>
       <c r="E22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J22">
         <v>3</v>
@@ -2931,19 +2931,19 @@
         <v>124</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J23">
         <v>2</v>
@@ -3260,19 +3260,19 @@
         <v>131</v>
       </c>
       <c r="E30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J30">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>5</v>
       </c>
       <c r="F31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G31">
         <v>5</v>
@@ -3354,16 +3354,16 @@
         <v>133</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G32">
         <v>5</v>
       </c>
       <c r="H32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I32">
         <v>5</v>
@@ -3404,7 +3404,7 @@
         <v>5</v>
       </c>
       <c r="F33">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G33">
         <v>5</v>
@@ -3545,16 +3545,16 @@
         <v>5</v>
       </c>
       <c r="F36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H36">
         <v>5</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J36">
         <v>4</v>
@@ -3824,19 +3824,19 @@
         <v>143</v>
       </c>
       <c r="E42">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I42">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J42">
         <v>3</v>
@@ -3871,16 +3871,16 @@
         <v>144</v>
       </c>
       <c r="E43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G43">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I43">
         <v>5</v>
@@ -4106,16 +4106,16 @@
         <v>149</v>
       </c>
       <c r="E48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G48">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I48">
         <v>5</v>
@@ -4262,7 +4262,7 @@
         <v>2</v>
       </c>
       <c r="J51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K51">
         <v>5</v>
@@ -4271,10 +4271,10 @@
         <v>5</v>
       </c>
       <c r="M51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O51">
         <v>6</v>
@@ -4294,16 +4294,16 @@
         <v>153</v>
       </c>
       <c r="E52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F52">
         <v>5</v>
       </c>
       <c r="G52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I52">
         <v>5</v>
@@ -4341,19 +4341,19 @@
         <v>154</v>
       </c>
       <c r="E53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J53">
         <v>3</v>
@@ -4400,7 +4400,7 @@
         <v>5</v>
       </c>
       <c r="I54">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>3</v>
@@ -4441,13 +4441,13 @@
         <v>5</v>
       </c>
       <c r="G55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H55">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>1</v>
@@ -4491,7 +4491,7 @@
         <v>5</v>
       </c>
       <c r="H56">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I56">
         <v>5</v>
@@ -4600,7 +4600,7 @@
         <v>4</v>
       </c>
       <c r="M58">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N58">
         <v>4</v>
@@ -4717,19 +4717,19 @@
         <v>162</v>
       </c>
       <c r="E61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -4867,7 +4867,7 @@
         <v>5</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I64">
         <v>4</v>
@@ -4905,19 +4905,19 @@
         <v>166</v>
       </c>
       <c r="E65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J65">
         <v>2</v>
@@ -5296,19 +5296,19 @@
         <v>2</v>
       </c>
       <c r="J73">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L73">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5375,19 +5375,19 @@
         <v>176</v>
       </c>
       <c r="E75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F75">
         <v>5</v>
       </c>
       <c r="G75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H75">
         <v>5</v>
       </c>
       <c r="I75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J75">
         <v>4</v>
@@ -5487,13 +5487,13 @@
         <v>5</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L77">
         <v>5</v>
       </c>
       <c r="M77">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N77">
         <v>4</v>
@@ -5516,19 +5516,19 @@
         <v>179</v>
       </c>
       <c r="E78">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H78">
         <v>5</v>
       </c>
       <c r="I78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J78">
         <v>3</v>
@@ -5569,7 +5569,7 @@
         <v>4</v>
       </c>
       <c r="G79">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H79">
         <v>4</v>
@@ -5716,7 +5716,7 @@
         <v>4</v>
       </c>
       <c r="I82">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J82">
         <v>3</v>
@@ -5848,7 +5848,7 @@
         <v>4</v>
       </c>
       <c r="F85">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G85">
         <v>4</v>
@@ -5901,7 +5901,7 @@
         <v>5</v>
       </c>
       <c r="H86">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I86">
         <v>4</v>
@@ -5998,7 +5998,7 @@
         <v>4</v>
       </c>
       <c r="I88">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J88">
         <v>4</v>
@@ -6080,19 +6080,19 @@
         <v>191</v>
       </c>
       <c r="E90">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F90">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G90">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H90">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I90">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J90">
         <v>2</v>
@@ -6174,19 +6174,19 @@
         <v>193</v>
       </c>
       <c r="E92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F92">
         <v>5</v>
       </c>
       <c r="G92">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J92">
         <v>1</v>
@@ -6268,16 +6268,16 @@
         <v>195</v>
       </c>
       <c r="E94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G94">
         <v>5</v>
       </c>
       <c r="H94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I94">
         <v>5</v>
@@ -6289,10 +6289,10 @@
         <v>5</v>
       </c>
       <c r="L94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N94">
         <v>5</v>
@@ -6459,13 +6459,13 @@
         <v>5</v>
       </c>
       <c r="F98">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G98">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H98">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I98">
         <v>5</v>
@@ -6506,7 +6506,7 @@
         <v>5</v>
       </c>
       <c r="F99">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G99">
         <v>5</v>
@@ -6615,7 +6615,7 @@
         <v>4</v>
       </c>
       <c r="K101">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L101">
         <v>4</v>
@@ -6741,7 +6741,7 @@
         <v>5</v>
       </c>
       <c r="F104">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G104">
         <v>5</v>
@@ -6841,10 +6841,10 @@
         <v>5</v>
       </c>
       <c r="H106">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I106">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J106">
         <v>3</v>
@@ -6926,16 +6926,16 @@
         <v>209</v>
       </c>
       <c r="E108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G108">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I108">
         <v>5</v>
@@ -6973,10 +6973,10 @@
         <v>210</v>
       </c>
       <c r="E109">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F109">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G109">
         <v>4</v>
@@ -7020,19 +7020,19 @@
         <v>211</v>
       </c>
       <c r="E110">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J110">
         <v>4</v>
@@ -7114,7 +7114,7 @@
         <v>213</v>
       </c>
       <c r="E112">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F112">
         <v>5</v>
@@ -7164,16 +7164,16 @@
         <v>5</v>
       </c>
       <c r="F113">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G113">
         <v>5</v>
       </c>
       <c r="H113">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I113">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J113">
         <v>1</v>
@@ -7267,7 +7267,7 @@
         <v>4</v>
       </c>
       <c r="I115">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J115">
         <v>4</v>
@@ -7308,7 +7308,7 @@
         <v>5</v>
       </c>
       <c r="G116">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116">
         <v>5</v>
@@ -7317,7 +7317,7 @@
         <v>5</v>
       </c>
       <c r="J116">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K116">
         <v>4</v>
@@ -7349,19 +7349,19 @@
         <v>218</v>
       </c>
       <c r="E117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F117">
         <v>5</v>
       </c>
       <c r="G117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H117">
         <v>5</v>
       </c>
       <c r="I117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J117">
         <v>2</v>
@@ -7396,19 +7396,19 @@
         <v>219</v>
       </c>
       <c r="E118">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F118">
         <v>5</v>
       </c>
       <c r="G118">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H118">
         <v>5</v>
       </c>
       <c r="I118">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J118">
         <v>4</v>
@@ -7493,7 +7493,7 @@
         <v>5</v>
       </c>
       <c r="F120">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G120">
         <v>5</v>
@@ -7584,19 +7584,19 @@
         <v>223</v>
       </c>
       <c r="E122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F122">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I122">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J122">
         <v>1</v>
@@ -7775,7 +7775,7 @@
         <v>4</v>
       </c>
       <c r="F126">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G126">
         <v>5</v>
@@ -7872,13 +7872,13 @@
         <v>5</v>
       </c>
       <c r="G128">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H128">
         <v>5</v>
       </c>
       <c r="I128">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J128">
         <v>3</v>
@@ -7913,19 +7913,19 @@
         <v>230</v>
       </c>
       <c r="E129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F129">
         <v>5</v>
       </c>
       <c r="G129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J129">
         <v>1</v>
@@ -8013,10 +8013,10 @@
         <v>4</v>
       </c>
       <c r="G131">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H131">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I131">
         <v>5</v>
@@ -8242,19 +8242,19 @@
         <v>237</v>
       </c>
       <c r="E136">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F136">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G136">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H136">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I136">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J136">
         <v>3</v>
@@ -8298,10 +8298,10 @@
         <v>5</v>
       </c>
       <c r="H137">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I137">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J137">
         <v>3</v>
@@ -8336,13 +8336,13 @@
         <v>239</v>
       </c>
       <c r="E138">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F138">
         <v>5</v>
       </c>
       <c r="G138">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H138">
         <v>5</v>
@@ -8386,7 +8386,7 @@
         <v>5</v>
       </c>
       <c r="F139">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G139">
         <v>5</v>
@@ -8477,19 +8477,19 @@
         <v>242</v>
       </c>
       <c r="E141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J141">
         <v>1</v>
@@ -8524,16 +8524,16 @@
         <v>243</v>
       </c>
       <c r="E142">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F142">
         <v>5</v>
       </c>
       <c r="G142">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H142">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I142">
         <v>5</v>
@@ -8639,7 +8639,7 @@
         <v>4</v>
       </c>
       <c r="L144">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M144">
         <v>4</v>
@@ -8900,19 +8900,19 @@
         <v>251</v>
       </c>
       <c r="E150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F150">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G150">
         <v>5</v>
       </c>
       <c r="H150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J150">
         <v>2</v>
@@ -8950,7 +8950,7 @@
         <v>5</v>
       </c>
       <c r="F151">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G151">
         <v>4</v>
@@ -9015,7 +9015,7 @@
         <v>3</v>
       </c>
       <c r="L152">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M152">
         <v>5</v>
@@ -9041,19 +9041,19 @@
         <v>254</v>
       </c>
       <c r="E153">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H153">
         <v>5</v>
       </c>
       <c r="I153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J153">
         <v>2</v>
@@ -9088,19 +9088,19 @@
         <v>255</v>
       </c>
       <c r="E154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G154">
         <v>5</v>
       </c>
       <c r="H154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J154">
         <v>3</v>
@@ -9276,19 +9276,19 @@
         <v>259</v>
       </c>
       <c r="E158">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F158">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G158">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H158">
         <v>5</v>
       </c>
       <c r="I158">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J158">
         <v>2</v>
@@ -9417,19 +9417,19 @@
         <v>262</v>
       </c>
       <c r="E161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J161">
         <v>4</v>
@@ -9473,7 +9473,7 @@
         <v>5</v>
       </c>
       <c r="H162">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I162">
         <v>5</v>
@@ -9485,7 +9485,7 @@
         <v>5</v>
       </c>
       <c r="L162">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M162">
         <v>5</v>
@@ -9558,7 +9558,7 @@
         <v>265</v>
       </c>
       <c r="E164">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F164">
         <v>4</v>
@@ -9567,7 +9567,7 @@
         <v>5</v>
       </c>
       <c r="H164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I164">
         <v>5</v>
@@ -9579,10 +9579,10 @@
         <v>4</v>
       </c>
       <c r="L164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N164">
         <v>4</v>
@@ -9652,19 +9652,19 @@
         <v>267</v>
       </c>
       <c r="E166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J166">
         <v>1</v>
@@ -9699,19 +9699,19 @@
         <v>268</v>
       </c>
       <c r="E167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F167">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J167">
         <v>2</v>
@@ -9840,7 +9840,7 @@
         <v>271</v>
       </c>
       <c r="E170">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F170">
         <v>5</v>
@@ -9849,7 +9849,7 @@
         <v>5</v>
       </c>
       <c r="H170">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I170">
         <v>5</v>
@@ -9984,7 +9984,7 @@
         <v>4</v>
       </c>
       <c r="F173">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G173">
         <v>5</v>
@@ -10075,10 +10075,10 @@
         <v>276</v>
       </c>
       <c r="E175">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G175">
         <v>5</v>
@@ -10087,7 +10087,7 @@
         <v>5</v>
       </c>
       <c r="I175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J175">
         <v>4</v>
@@ -10096,7 +10096,7 @@
         <v>3</v>
       </c>
       <c r="L175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M175">
         <v>5</v>
@@ -10216,19 +10216,19 @@
         <v>279</v>
       </c>
       <c r="E178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F178">
         <v>5</v>
       </c>
       <c r="G178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J178">
         <v>1</v>
@@ -10266,10 +10266,10 @@
         <v>5</v>
       </c>
       <c r="F179">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G179">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H179">
         <v>5</v>
@@ -10357,7 +10357,7 @@
         <v>282</v>
       </c>
       <c r="E181">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F181">
         <v>4</v>
@@ -10545,19 +10545,19 @@
         <v>286</v>
       </c>
       <c r="E185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J185">
         <v>2</v>
@@ -10686,19 +10686,19 @@
         <v>289</v>
       </c>
       <c r="E188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H188">
         <v>5</v>
       </c>
       <c r="I188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J188">
         <v>1</v>
@@ -10748,19 +10748,19 @@
         <v>4</v>
       </c>
       <c r="J189">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K189">
         <v>5</v>
       </c>
       <c r="L189">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M189">
         <v>5</v>
       </c>
       <c r="N189">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O189">
         <v>6</v>
@@ -10780,19 +10780,19 @@
         <v>291</v>
       </c>
       <c r="E190">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F190">
         <v>5</v>
       </c>
       <c r="G190">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H190">
         <v>5</v>
       </c>
       <c r="I190">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J190">
         <v>3</v>
@@ -10842,19 +10842,19 @@
         <v>3</v>
       </c>
       <c r="J191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O191">
         <v>6</v>
@@ -10883,7 +10883,7 @@
         <v>5</v>
       </c>
       <c r="H192">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I192">
         <v>5</v>
@@ -10971,7 +10971,7 @@
         <v>5</v>
       </c>
       <c r="F194">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G194">
         <v>5</v>
@@ -11109,19 +11109,19 @@
         <v>298</v>
       </c>
       <c r="E197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G197">
         <v>5</v>
       </c>
       <c r="H197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J197">
         <v>4</v>
@@ -11168,7 +11168,7 @@
         <v>5</v>
       </c>
       <c r="I198">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J198">
         <v>2</v>
@@ -11259,7 +11259,7 @@
         <v>5</v>
       </c>
       <c r="H200">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I200">
         <v>5</v>
@@ -11488,10 +11488,10 @@
         <v>5</v>
       </c>
       <c r="F205">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G205">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H205">
         <v>5</v>
@@ -11579,19 +11579,19 @@
         <v>308</v>
       </c>
       <c r="E207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H207">
         <v>5</v>
       </c>
       <c r="I207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J207">
         <v>1</v>
@@ -11629,31 +11629,31 @@
         <v>5</v>
       </c>
       <c r="F208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K208">
         <v>4</v>
       </c>
       <c r="L208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O208">
         <v>6</v>
@@ -11676,16 +11676,16 @@
         <v>5</v>
       </c>
       <c r="F209">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G209">
         <v>5</v>
       </c>
       <c r="H209">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I209">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J209">
         <v>2</v>
@@ -11767,7 +11767,7 @@
         <v>312</v>
       </c>
       <c r="E211">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F211">
         <v>4</v>
@@ -11776,10 +11776,10 @@
         <v>5</v>
       </c>
       <c r="H211">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I211">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J211">
         <v>3</v>
@@ -11961,13 +11961,13 @@
         <v>4</v>
       </c>
       <c r="G215">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H215">
         <v>5</v>
       </c>
       <c r="I215">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J215">
         <v>2</v>
@@ -12014,7 +12014,7 @@
         <v>5</v>
       </c>
       <c r="I216">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J216">
         <v>1</v>
@@ -12152,10 +12152,10 @@
         <v>5</v>
       </c>
       <c r="H219">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I219">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J219">
         <v>3</v>
@@ -12202,7 +12202,7 @@
         <v>5</v>
       </c>
       <c r="I220">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J220">
         <v>3</v>
@@ -12249,7 +12249,7 @@
         <v>4</v>
       </c>
       <c r="I221">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J221">
         <v>2</v>
@@ -12331,19 +12331,19 @@
         <v>324</v>
       </c>
       <c r="E223">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J223">
         <v>3</v>
@@ -12519,19 +12519,19 @@
         <v>328</v>
       </c>
       <c r="E227">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F227">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G227">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H227">
         <v>5</v>
       </c>
       <c r="I227">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J227">
         <v>2</v>
@@ -12566,13 +12566,13 @@
         <v>329</v>
       </c>
       <c r="E228">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F228">
         <v>5</v>
       </c>
       <c r="G228">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H228">
         <v>5</v>
@@ -12663,10 +12663,10 @@
         <v>4</v>
       </c>
       <c r="F230">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G230">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H230">
         <v>5</v>
@@ -12707,19 +12707,19 @@
         <v>332</v>
       </c>
       <c r="E231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J231">
         <v>3</v>
@@ -12754,19 +12754,19 @@
         <v>333</v>
       </c>
       <c r="E232">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F232">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G232">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H232">
         <v>5</v>
       </c>
       <c r="I232">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J232">
         <v>2</v>
@@ -12989,19 +12989,19 @@
         <v>338</v>
       </c>
       <c r="E237">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F237">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G237">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H237">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I237">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J237">
         <v>1</v>
@@ -13048,7 +13048,7 @@
         <v>5</v>
       </c>
       <c r="I238">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J238">
         <v>3</v>
@@ -13130,19 +13130,19 @@
         <v>341</v>
       </c>
       <c r="E240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J240">
         <v>2</v>
@@ -13224,16 +13224,16 @@
         <v>343</v>
       </c>
       <c r="E242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I242">
         <v>5</v>
@@ -13298,7 +13298,7 @@
         <v>4</v>
       </c>
       <c r="N243">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O243">
         <v>6</v>
@@ -13318,19 +13318,19 @@
         <v>345</v>
       </c>
       <c r="E244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F244">
         <v>5</v>
       </c>
       <c r="G244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J244">
         <v>3</v>
@@ -13459,10 +13459,10 @@
         <v>348</v>
       </c>
       <c r="E247">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F247">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G247">
         <v>5</v>
@@ -13600,7 +13600,7 @@
         <v>351</v>
       </c>
       <c r="E250">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F250">
         <v>5</v>
@@ -13662,19 +13662,19 @@
         <v>4</v>
       </c>
       <c r="J251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L251">
         <v>5</v>
       </c>
       <c r="M251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O251">
         <v>6</v>
@@ -13844,7 +13844,7 @@
         <v>5</v>
       </c>
       <c r="H255">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I255">
         <v>5</v>
@@ -13929,7 +13929,7 @@
         <v>358</v>
       </c>
       <c r="E257">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F257">
         <v>5</v>
@@ -13941,7 +13941,7 @@
         <v>5</v>
       </c>
       <c r="I257">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J257">
         <v>4</v>
@@ -13976,16 +13976,16 @@
         <v>359</v>
       </c>
       <c r="E258">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F258">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G258">
         <v>5</v>
       </c>
       <c r="H258">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I258">
         <v>5</v>
@@ -14026,10 +14026,10 @@
         <v>5</v>
       </c>
       <c r="F259">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G259">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H259">
         <v>4</v>
@@ -14091,13 +14091,13 @@
         <v>4</v>
       </c>
       <c r="L260">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M260">
         <v>5</v>
       </c>
       <c r="N260">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O260">
         <v>6</v>
@@ -14211,19 +14211,19 @@
         <v>364</v>
       </c>
       <c r="E263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F263">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J263">
         <v>2</v>
@@ -14305,16 +14305,16 @@
         <v>366</v>
       </c>
       <c r="E265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I265">
         <v>5</v>
@@ -14467,13 +14467,13 @@
         <v>5</v>
       </c>
       <c r="L268">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M268">
         <v>5</v>
       </c>
       <c r="N268">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O268">
         <v>6</v>
@@ -14493,19 +14493,19 @@
         <v>370</v>
       </c>
       <c r="E269">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F269">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G269">
         <v>5</v>
       </c>
       <c r="H269">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I269">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J269">
         <v>2</v>
@@ -14552,7 +14552,7 @@
         <v>5</v>
       </c>
       <c r="I270">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J270">
         <v>3</v>
@@ -14614,7 +14614,7 @@
         <v>4</v>
       </c>
       <c r="N271">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O271">
         <v>6</v>
@@ -14643,7 +14643,7 @@
         <v>5</v>
       </c>
       <c r="H272">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I272">
         <v>5</v>
@@ -14681,7 +14681,7 @@
         <v>374</v>
       </c>
       <c r="E273">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F273">
         <v>5</v>
@@ -14837,16 +14837,16 @@
         <v>4</v>
       </c>
       <c r="J276">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K276">
         <v>5</v>
       </c>
       <c r="L276">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M276">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N276">
         <v>5</v>
@@ -14869,7 +14869,7 @@
         <v>378</v>
       </c>
       <c r="E277">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F277">
         <v>5</v>
@@ -15107,16 +15107,16 @@
         <v>5</v>
       </c>
       <c r="F282">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G282">
         <v>5</v>
       </c>
       <c r="H282">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I282">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J282">
         <v>4</v>
@@ -15178,7 +15178,7 @@
         <v>5</v>
       </c>
       <c r="N283">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O283">
         <v>6</v>
@@ -15351,7 +15351,7 @@
         <v>5</v>
       </c>
       <c r="I287">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J287">
         <v>3</v>
@@ -15386,19 +15386,19 @@
         <v>389</v>
       </c>
       <c r="E288">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F288">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G288">
         <v>5</v>
       </c>
       <c r="H288">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I288">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J288">
         <v>3</v>
@@ -15721,10 +15721,10 @@
         <v>5</v>
       </c>
       <c r="G295">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H295">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I295">
         <v>5</v>
@@ -15856,19 +15856,19 @@
         <v>399</v>
       </c>
       <c r="E298">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H298">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J298">
         <v>3</v>
@@ -15903,16 +15903,16 @@
         <v>400</v>
       </c>
       <c r="E299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I299">
         <v>5</v>
@@ -16006,7 +16006,7 @@
         <v>4</v>
       </c>
       <c r="H301">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I301">
         <v>5</v>
@@ -16044,13 +16044,13 @@
         <v>403</v>
       </c>
       <c r="E302">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F302">
         <v>5</v>
       </c>
       <c r="G302">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H302">
         <v>5</v>
@@ -16091,7 +16091,7 @@
         <v>404</v>
       </c>
       <c r="E303">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F303">
         <v>5</v>
@@ -16326,19 +16326,19 @@
         <v>409</v>
       </c>
       <c r="E308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H308">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J308">
         <v>1</v>
@@ -16467,16 +16467,16 @@
         <v>412</v>
       </c>
       <c r="E311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G311">
         <v>5</v>
       </c>
       <c r="H311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I311">
         <v>5</v>
@@ -16567,7 +16567,7 @@
         <v>5</v>
       </c>
       <c r="G313">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H313">
         <v>5</v>
@@ -16702,19 +16702,19 @@
         <v>417</v>
       </c>
       <c r="E316">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F316">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G316">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H316">
         <v>5</v>
       </c>
       <c r="I316">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J316">
         <v>2</v>
@@ -16749,16 +16749,16 @@
         <v>418</v>
       </c>
       <c r="E317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I317">
         <v>5</v>
@@ -16796,7 +16796,7 @@
         <v>419</v>
       </c>
       <c r="E318">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F318">
         <v>5</v>
@@ -16808,7 +16808,7 @@
         <v>5</v>
       </c>
       <c r="I318">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J318">
         <v>1</v>
@@ -16843,16 +16843,16 @@
         <v>420</v>
       </c>
       <c r="E319">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F319">
         <v>5</v>
       </c>
       <c r="G319">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H319">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I319">
         <v>5</v>
@@ -16890,19 +16890,19 @@
         <v>421</v>
       </c>
       <c r="E320">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F320">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G320">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H320">
         <v>5</v>
       </c>
       <c r="I320">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J320">
         <v>2</v>
@@ -17219,7 +17219,7 @@
         <v>428</v>
       </c>
       <c r="E327">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F327">
         <v>5</v>
@@ -17269,7 +17269,7 @@
         <v>4</v>
       </c>
       <c r="F328">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G328">
         <v>5</v>
@@ -17313,19 +17313,19 @@
         <v>430</v>
       </c>
       <c r="E329">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F329">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G329">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H329">
         <v>5</v>
       </c>
       <c r="I329">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J329">
         <v>3</v>
@@ -17454,19 +17454,19 @@
         <v>433</v>
       </c>
       <c r="E332">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F332">
         <v>5</v>
       </c>
       <c r="G332">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H332">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I332">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J332">
         <v>4</v>
@@ -17595,19 +17595,19 @@
         <v>436</v>
       </c>
       <c r="E335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G335">
         <v>4</v>
       </c>
       <c r="H335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J335">
         <v>1</v>
@@ -17836,7 +17836,7 @@
         <v>5</v>
       </c>
       <c r="G340">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H340">
         <v>5</v>
@@ -17877,7 +17877,7 @@
         <v>442</v>
       </c>
       <c r="E341">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F341">
         <v>4</v>
@@ -17886,7 +17886,7 @@
         <v>4</v>
       </c>
       <c r="H341">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I341">
         <v>5</v>
@@ -17924,19 +17924,19 @@
         <v>443</v>
       </c>
       <c r="E342">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F342">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G342">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H342">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I342">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J342">
         <v>1</v>
@@ -18071,7 +18071,7 @@
         <v>4</v>
       </c>
       <c r="G345">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H345">
         <v>4</v>
@@ -18115,7 +18115,7 @@
         <v>4</v>
       </c>
       <c r="F346">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G346">
         <v>5</v>
@@ -18206,19 +18206,19 @@
         <v>449</v>
       </c>
       <c r="E348">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H348">
         <v>5</v>
       </c>
       <c r="I348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J348">
         <v>2</v>
@@ -18300,19 +18300,19 @@
         <v>451</v>
       </c>
       <c r="E350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H350">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J350">
         <v>4</v>
@@ -18347,7 +18347,7 @@
         <v>452</v>
       </c>
       <c r="E351">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F351">
         <v>5</v>
@@ -18356,7 +18356,7 @@
         <v>5</v>
       </c>
       <c r="H351">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I351">
         <v>5</v>
@@ -18400,7 +18400,7 @@
         <v>5</v>
       </c>
       <c r="G352">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H352">
         <v>5</v>
@@ -18488,19 +18488,19 @@
         <v>455</v>
       </c>
       <c r="E354">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F354">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G354">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H354">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I354">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J354">
         <v>4</v>
@@ -18535,19 +18535,19 @@
         <v>456</v>
       </c>
       <c r="E355">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F355">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G355">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H355">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I355">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J355">
         <v>1</v>
@@ -18629,19 +18629,19 @@
         <v>458</v>
       </c>
       <c r="E357">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F357">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G357">
         <v>5</v>
       </c>
       <c r="H357">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I357">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J357">
         <v>2</v>
@@ -18723,7 +18723,7 @@
         <v>460</v>
       </c>
       <c r="E359">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F359">
         <v>5</v>
@@ -18732,10 +18732,10 @@
         <v>5</v>
       </c>
       <c r="H359">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I359">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J359">
         <v>3</v>
@@ -18829,7 +18829,7 @@
         <v>5</v>
       </c>
       <c r="I361">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J361">
         <v>3</v>
@@ -18864,7 +18864,7 @@
         <v>463</v>
       </c>
       <c r="E362">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F362">
         <v>5</v>
@@ -19005,19 +19005,19 @@
         <v>466</v>
       </c>
       <c r="E365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H365">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J365">
         <v>1</v>
@@ -19052,7 +19052,7 @@
         <v>467</v>
       </c>
       <c r="E366">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F366">
         <v>5</v>
@@ -19108,7 +19108,7 @@
         <v>5</v>
       </c>
       <c r="H367">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I367">
         <v>5</v>
@@ -19146,7 +19146,7 @@
         <v>469</v>
       </c>
       <c r="E368">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F368">
         <v>5</v>
@@ -19199,7 +19199,7 @@
         <v>5</v>
       </c>
       <c r="G369">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H369">
         <v>4</v>
@@ -19340,7 +19340,7 @@
         <v>4</v>
       </c>
       <c r="G372">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H372">
         <v>4</v>
@@ -19475,7 +19475,7 @@
         <v>476</v>
       </c>
       <c r="E375">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F375">
         <v>5</v>
@@ -19522,19 +19522,19 @@
         <v>477</v>
       </c>
       <c r="E376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G376">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J376">
         <v>4</v>
@@ -19713,7 +19713,7 @@
         <v>5</v>
       </c>
       <c r="F380">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G380">
         <v>5</v>
@@ -19757,13 +19757,13 @@
         <v>482</v>
       </c>
       <c r="E381">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F381">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G381">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H381">
         <v>5</v>
@@ -19804,16 +19804,16 @@
         <v>483</v>
       </c>
       <c r="E382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F382">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G382">
         <v>5</v>
       </c>
       <c r="H382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I382">
         <v>5</v>
@@ -19898,19 +19898,19 @@
         <v>485</v>
       </c>
       <c r="E384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J384">
         <v>3</v>
@@ -19992,19 +19992,19 @@
         <v>487</v>
       </c>
       <c r="E386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H386">
         <v>5</v>
       </c>
       <c r="I386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J386">
         <v>3</v>
@@ -20327,10 +20327,10 @@
         <v>5</v>
       </c>
       <c r="G393">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H393">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I393">
         <v>5</v>
@@ -20421,7 +20421,7 @@
         <v>4</v>
       </c>
       <c r="G395">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H395">
         <v>3</v>
@@ -20486,10 +20486,10 @@
         <v>4</v>
       </c>
       <c r="M396">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N396">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O396">
         <v>6</v>
@@ -20512,16 +20512,16 @@
         <v>5</v>
       </c>
       <c r="F397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J397">
         <v>2</v>
@@ -20650,7 +20650,7 @@
         <v>501</v>
       </c>
       <c r="E400">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F400">
         <v>5</v>
@@ -20659,10 +20659,10 @@
         <v>5</v>
       </c>
       <c r="H400">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I400">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J400">
         <v>4</v>
@@ -20712,7 +20712,7 @@
         <v>4</v>
       </c>
       <c r="J401">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K401">
         <v>5</v>

</xml_diff>

<commit_message>
delivery v3.5: full 1-7 Likert range; Table 1A df=539 for 7-factor
</commit_message>
<xml_diff>
--- a/data/T2_cleaned.xlsx
+++ b/data/T2_cleaned.xlsx
@@ -1968,7 +1968,7 @@
         <v>5</v>
       </c>
       <c r="M2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N2">
         <v>5</v>
@@ -1991,7 +1991,7 @@
         <v>104</v>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2009,7 +2009,7 @@
         <v>4</v>
       </c>
       <c r="K3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L3">
         <v>4</v>
@@ -2367,7 +2367,7 @@
         <v>112</v>
       </c>
       <c r="E11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F11">
         <v>5</v>
@@ -2379,7 +2379,7 @@
         <v>5</v>
       </c>
       <c r="I11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J11">
         <v>2</v>
@@ -2414,19 +2414,19 @@
         <v>113</v>
       </c>
       <c r="E12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J12">
         <v>2</v>
@@ -2461,19 +2461,19 @@
         <v>114</v>
       </c>
       <c r="E13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J13">
         <v>2</v>
@@ -2517,7 +2517,7 @@
         <v>5</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I14">
         <v>4</v>
@@ -2790,19 +2790,19 @@
         <v>121</v>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J20">
         <v>3</v>
@@ -2884,19 +2884,19 @@
         <v>123</v>
       </c>
       <c r="E22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J22">
         <v>3</v>
@@ -2931,19 +2931,19 @@
         <v>124</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J23">
         <v>2</v>
@@ -3260,19 +3260,19 @@
         <v>131</v>
       </c>
       <c r="E30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J30">
         <v>4</v>
@@ -3310,7 +3310,7 @@
         <v>5</v>
       </c>
       <c r="F31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G31">
         <v>5</v>
@@ -3354,16 +3354,16 @@
         <v>133</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G32">
         <v>5</v>
       </c>
       <c r="H32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I32">
         <v>5</v>
@@ -3404,7 +3404,7 @@
         <v>5</v>
       </c>
       <c r="F33">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G33">
         <v>5</v>
@@ -3545,16 +3545,16 @@
         <v>5</v>
       </c>
       <c r="F36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H36">
         <v>5</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J36">
         <v>4</v>
@@ -3824,19 +3824,19 @@
         <v>143</v>
       </c>
       <c r="E42">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I42">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J42">
         <v>3</v>
@@ -3871,16 +3871,16 @@
         <v>144</v>
       </c>
       <c r="E43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G43">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I43">
         <v>5</v>
@@ -4106,16 +4106,16 @@
         <v>149</v>
       </c>
       <c r="E48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G48">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I48">
         <v>5</v>
@@ -4262,7 +4262,7 @@
         <v>2</v>
       </c>
       <c r="J51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K51">
         <v>5</v>
@@ -4271,10 +4271,10 @@
         <v>5</v>
       </c>
       <c r="M51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O51">
         <v>6</v>
@@ -4294,16 +4294,16 @@
         <v>153</v>
       </c>
       <c r="E52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F52">
         <v>5</v>
       </c>
       <c r="G52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H52">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I52">
         <v>5</v>
@@ -4341,19 +4341,19 @@
         <v>154</v>
       </c>
       <c r="E53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J53">
         <v>3</v>
@@ -4400,7 +4400,7 @@
         <v>5</v>
       </c>
       <c r="I54">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>3</v>
@@ -4441,13 +4441,13 @@
         <v>5</v>
       </c>
       <c r="G55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H55">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J55">
         <v>1</v>
@@ -4491,7 +4491,7 @@
         <v>5</v>
       </c>
       <c r="H56">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I56">
         <v>5</v>
@@ -4600,7 +4600,7 @@
         <v>4</v>
       </c>
       <c r="M58">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N58">
         <v>4</v>
@@ -4717,19 +4717,19 @@
         <v>162</v>
       </c>
       <c r="E61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I61">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J61">
         <v>3</v>
@@ -4867,7 +4867,7 @@
         <v>5</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I64">
         <v>4</v>
@@ -4905,19 +4905,19 @@
         <v>166</v>
       </c>
       <c r="E65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J65">
         <v>2</v>
@@ -5296,19 +5296,19 @@
         <v>2</v>
       </c>
       <c r="J73">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L73">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5375,19 +5375,19 @@
         <v>176</v>
       </c>
       <c r="E75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F75">
         <v>5</v>
       </c>
       <c r="G75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H75">
         <v>5</v>
       </c>
       <c r="I75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J75">
         <v>4</v>
@@ -5487,13 +5487,13 @@
         <v>5</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L77">
         <v>5</v>
       </c>
       <c r="M77">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N77">
         <v>4</v>
@@ -5516,19 +5516,19 @@
         <v>179</v>
       </c>
       <c r="E78">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H78">
         <v>5</v>
       </c>
       <c r="I78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J78">
         <v>3</v>
@@ -5569,7 +5569,7 @@
         <v>4</v>
       </c>
       <c r="G79">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H79">
         <v>4</v>
@@ -5716,7 +5716,7 @@
         <v>4</v>
       </c>
       <c r="I82">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J82">
         <v>3</v>
@@ -5848,7 +5848,7 @@
         <v>4</v>
       </c>
       <c r="F85">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G85">
         <v>4</v>
@@ -5901,7 +5901,7 @@
         <v>5</v>
       </c>
       <c r="H86">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I86">
         <v>4</v>
@@ -5998,7 +5998,7 @@
         <v>4</v>
       </c>
       <c r="I88">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J88">
         <v>4</v>
@@ -6080,19 +6080,19 @@
         <v>191</v>
       </c>
       <c r="E90">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F90">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G90">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H90">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I90">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J90">
         <v>2</v>
@@ -6174,19 +6174,19 @@
         <v>193</v>
       </c>
       <c r="E92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F92">
         <v>5</v>
       </c>
       <c r="G92">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I92">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J92">
         <v>1</v>
@@ -6268,16 +6268,16 @@
         <v>195</v>
       </c>
       <c r="E94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G94">
         <v>5</v>
       </c>
       <c r="H94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I94">
         <v>5</v>
@@ -6289,10 +6289,10 @@
         <v>5</v>
       </c>
       <c r="L94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M94">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N94">
         <v>5</v>
@@ -6459,13 +6459,13 @@
         <v>5</v>
       </c>
       <c r="F98">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G98">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H98">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I98">
         <v>5</v>
@@ -6506,7 +6506,7 @@
         <v>5</v>
       </c>
       <c r="F99">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G99">
         <v>5</v>
@@ -6615,7 +6615,7 @@
         <v>4</v>
       </c>
       <c r="K101">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L101">
         <v>4</v>
@@ -6741,7 +6741,7 @@
         <v>5</v>
       </c>
       <c r="F104">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G104">
         <v>5</v>
@@ -6841,10 +6841,10 @@
         <v>5</v>
       </c>
       <c r="H106">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I106">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J106">
         <v>3</v>
@@ -6926,16 +6926,16 @@
         <v>209</v>
       </c>
       <c r="E108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G108">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H108">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I108">
         <v>5</v>
@@ -6973,10 +6973,10 @@
         <v>210</v>
       </c>
       <c r="E109">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F109">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G109">
         <v>4</v>
@@ -7020,19 +7020,19 @@
         <v>211</v>
       </c>
       <c r="E110">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I110">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J110">
         <v>4</v>
@@ -7114,7 +7114,7 @@
         <v>213</v>
       </c>
       <c r="E112">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F112">
         <v>5</v>
@@ -7164,16 +7164,16 @@
         <v>5</v>
       </c>
       <c r="F113">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G113">
         <v>5</v>
       </c>
       <c r="H113">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I113">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J113">
         <v>1</v>
@@ -7267,7 +7267,7 @@
         <v>4</v>
       </c>
       <c r="I115">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J115">
         <v>4</v>
@@ -7308,7 +7308,7 @@
         <v>5</v>
       </c>
       <c r="G116">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H116">
         <v>5</v>
@@ -7317,7 +7317,7 @@
         <v>5</v>
       </c>
       <c r="J116">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K116">
         <v>4</v>
@@ -7349,19 +7349,19 @@
         <v>218</v>
       </c>
       <c r="E117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F117">
         <v>5</v>
       </c>
       <c r="G117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H117">
         <v>5</v>
       </c>
       <c r="I117">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J117">
         <v>2</v>
@@ -7396,19 +7396,19 @@
         <v>219</v>
       </c>
       <c r="E118">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F118">
         <v>5</v>
       </c>
       <c r="G118">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H118">
         <v>5</v>
       </c>
       <c r="I118">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J118">
         <v>4</v>
@@ -7493,7 +7493,7 @@
         <v>5</v>
       </c>
       <c r="F120">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G120">
         <v>5</v>
@@ -7584,19 +7584,19 @@
         <v>223</v>
       </c>
       <c r="E122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F122">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H122">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I122">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J122">
         <v>1</v>
@@ -7775,7 +7775,7 @@
         <v>4</v>
       </c>
       <c r="F126">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G126">
         <v>5</v>
@@ -7872,13 +7872,13 @@
         <v>5</v>
       </c>
       <c r="G128">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H128">
         <v>5</v>
       </c>
       <c r="I128">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J128">
         <v>3</v>
@@ -7913,19 +7913,19 @@
         <v>230</v>
       </c>
       <c r="E129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F129">
         <v>5</v>
       </c>
       <c r="G129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J129">
         <v>1</v>
@@ -8013,10 +8013,10 @@
         <v>4</v>
       </c>
       <c r="G131">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H131">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I131">
         <v>5</v>
@@ -8242,19 +8242,19 @@
         <v>237</v>
       </c>
       <c r="E136">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F136">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G136">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H136">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I136">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J136">
         <v>3</v>
@@ -8298,10 +8298,10 @@
         <v>5</v>
       </c>
       <c r="H137">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I137">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J137">
         <v>3</v>
@@ -8336,13 +8336,13 @@
         <v>239</v>
       </c>
       <c r="E138">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F138">
         <v>5</v>
       </c>
       <c r="G138">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H138">
         <v>5</v>
@@ -8386,7 +8386,7 @@
         <v>5</v>
       </c>
       <c r="F139">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G139">
         <v>5</v>
@@ -8477,19 +8477,19 @@
         <v>242</v>
       </c>
       <c r="E141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I141">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J141">
         <v>1</v>
@@ -8524,16 +8524,16 @@
         <v>243</v>
       </c>
       <c r="E142">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F142">
         <v>5</v>
       </c>
       <c r="G142">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H142">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I142">
         <v>5</v>
@@ -8639,7 +8639,7 @@
         <v>4</v>
       </c>
       <c r="L144">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M144">
         <v>4</v>
@@ -8900,19 +8900,19 @@
         <v>251</v>
       </c>
       <c r="E150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F150">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G150">
         <v>5</v>
       </c>
       <c r="H150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I150">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J150">
         <v>2</v>
@@ -8950,7 +8950,7 @@
         <v>5</v>
       </c>
       <c r="F151">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G151">
         <v>4</v>
@@ -9015,7 +9015,7 @@
         <v>3</v>
       </c>
       <c r="L152">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M152">
         <v>5</v>
@@ -9041,19 +9041,19 @@
         <v>254</v>
       </c>
       <c r="E153">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H153">
         <v>5</v>
       </c>
       <c r="I153">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J153">
         <v>2</v>
@@ -9088,19 +9088,19 @@
         <v>255</v>
       </c>
       <c r="E154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G154">
         <v>5</v>
       </c>
       <c r="H154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I154">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J154">
         <v>3</v>
@@ -9276,19 +9276,19 @@
         <v>259</v>
       </c>
       <c r="E158">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F158">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G158">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H158">
         <v>5</v>
       </c>
       <c r="I158">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J158">
         <v>2</v>
@@ -9417,19 +9417,19 @@
         <v>262</v>
       </c>
       <c r="E161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I161">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J161">
         <v>4</v>
@@ -9473,7 +9473,7 @@
         <v>5</v>
       </c>
       <c r="H162">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I162">
         <v>5</v>
@@ -9485,7 +9485,7 @@
         <v>5</v>
       </c>
       <c r="L162">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M162">
         <v>5</v>
@@ -9558,7 +9558,7 @@
         <v>265</v>
       </c>
       <c r="E164">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F164">
         <v>4</v>
@@ -9567,7 +9567,7 @@
         <v>5</v>
       </c>
       <c r="H164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I164">
         <v>5</v>
@@ -9579,10 +9579,10 @@
         <v>4</v>
       </c>
       <c r="L164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M164">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N164">
         <v>4</v>
@@ -9652,19 +9652,19 @@
         <v>267</v>
       </c>
       <c r="E166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I166">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J166">
         <v>1</v>
@@ -9699,19 +9699,19 @@
         <v>268</v>
       </c>
       <c r="E167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F167">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I167">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J167">
         <v>2</v>
@@ -9840,7 +9840,7 @@
         <v>271</v>
       </c>
       <c r="E170">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F170">
         <v>5</v>
@@ -9849,7 +9849,7 @@
         <v>5</v>
       </c>
       <c r="H170">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I170">
         <v>5</v>
@@ -9984,7 +9984,7 @@
         <v>4</v>
       </c>
       <c r="F173">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G173">
         <v>5</v>
@@ -10075,10 +10075,10 @@
         <v>276</v>
       </c>
       <c r="E175">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G175">
         <v>5</v>
@@ -10087,7 +10087,7 @@
         <v>5</v>
       </c>
       <c r="I175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J175">
         <v>4</v>
@@ -10096,7 +10096,7 @@
         <v>3</v>
       </c>
       <c r="L175">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M175">
         <v>5</v>
@@ -10216,19 +10216,19 @@
         <v>279</v>
       </c>
       <c r="E178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F178">
         <v>5</v>
       </c>
       <c r="G178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I178">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J178">
         <v>1</v>
@@ -10266,10 +10266,10 @@
         <v>5</v>
       </c>
       <c r="F179">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G179">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H179">
         <v>5</v>
@@ -10357,7 +10357,7 @@
         <v>282</v>
       </c>
       <c r="E181">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F181">
         <v>4</v>
@@ -10545,19 +10545,19 @@
         <v>286</v>
       </c>
       <c r="E185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I185">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J185">
         <v>2</v>
@@ -10686,19 +10686,19 @@
         <v>289</v>
       </c>
       <c r="E188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H188">
         <v>5</v>
       </c>
       <c r="I188">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J188">
         <v>1</v>
@@ -10748,19 +10748,19 @@
         <v>4</v>
       </c>
       <c r="J189">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K189">
         <v>5</v>
       </c>
       <c r="L189">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M189">
         <v>5</v>
       </c>
       <c r="N189">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O189">
         <v>6</v>
@@ -10780,19 +10780,19 @@
         <v>291</v>
       </c>
       <c r="E190">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F190">
         <v>5</v>
       </c>
       <c r="G190">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H190">
         <v>5</v>
       </c>
       <c r="I190">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J190">
         <v>3</v>
@@ -10842,19 +10842,19 @@
         <v>3</v>
       </c>
       <c r="J191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N191">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O191">
         <v>6</v>
@@ -10883,7 +10883,7 @@
         <v>5</v>
       </c>
       <c r="H192">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I192">
         <v>5</v>
@@ -10971,7 +10971,7 @@
         <v>5</v>
       </c>
       <c r="F194">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G194">
         <v>5</v>
@@ -11109,19 +11109,19 @@
         <v>298</v>
       </c>
       <c r="E197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G197">
         <v>5</v>
       </c>
       <c r="H197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I197">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J197">
         <v>4</v>
@@ -11168,7 +11168,7 @@
         <v>5</v>
       </c>
       <c r="I198">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J198">
         <v>2</v>
@@ -11259,7 +11259,7 @@
         <v>5</v>
       </c>
       <c r="H200">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I200">
         <v>5</v>
@@ -11488,10 +11488,10 @@
         <v>5</v>
       </c>
       <c r="F205">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G205">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H205">
         <v>5</v>
@@ -11579,19 +11579,19 @@
         <v>308</v>
       </c>
       <c r="E207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H207">
         <v>5</v>
       </c>
       <c r="I207">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J207">
         <v>1</v>
@@ -11629,31 +11629,31 @@
         <v>5</v>
       </c>
       <c r="F208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K208">
         <v>4</v>
       </c>
       <c r="L208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M208">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N208">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O208">
         <v>6</v>
@@ -11676,16 +11676,16 @@
         <v>5</v>
       </c>
       <c r="F209">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G209">
         <v>5</v>
       </c>
       <c r="H209">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I209">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J209">
         <v>2</v>
@@ -11767,7 +11767,7 @@
         <v>312</v>
       </c>
       <c r="E211">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F211">
         <v>4</v>
@@ -11776,10 +11776,10 @@
         <v>5</v>
       </c>
       <c r="H211">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I211">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J211">
         <v>3</v>
@@ -11961,13 +11961,13 @@
         <v>4</v>
       </c>
       <c r="G215">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H215">
         <v>5</v>
       </c>
       <c r="I215">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J215">
         <v>2</v>
@@ -12014,7 +12014,7 @@
         <v>5</v>
       </c>
       <c r="I216">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J216">
         <v>1</v>
@@ -12152,10 +12152,10 @@
         <v>5</v>
       </c>
       <c r="H219">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I219">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J219">
         <v>3</v>
@@ -12202,7 +12202,7 @@
         <v>5</v>
       </c>
       <c r="I220">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J220">
         <v>3</v>
@@ -12249,7 +12249,7 @@
         <v>4</v>
       </c>
       <c r="I221">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J221">
         <v>2</v>
@@ -12331,19 +12331,19 @@
         <v>324</v>
       </c>
       <c r="E223">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I223">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J223">
         <v>3</v>
@@ -12519,19 +12519,19 @@
         <v>328</v>
       </c>
       <c r="E227">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F227">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G227">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H227">
         <v>5</v>
       </c>
       <c r="I227">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J227">
         <v>2</v>
@@ -12566,13 +12566,13 @@
         <v>329</v>
       </c>
       <c r="E228">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F228">
         <v>5</v>
       </c>
       <c r="G228">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H228">
         <v>5</v>
@@ -12663,10 +12663,10 @@
         <v>4</v>
       </c>
       <c r="F230">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G230">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H230">
         <v>5</v>
@@ -12707,19 +12707,19 @@
         <v>332</v>
       </c>
       <c r="E231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I231">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J231">
         <v>3</v>
@@ -12754,19 +12754,19 @@
         <v>333</v>
       </c>
       <c r="E232">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F232">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G232">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H232">
         <v>5</v>
       </c>
       <c r="I232">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J232">
         <v>2</v>
@@ -12989,19 +12989,19 @@
         <v>338</v>
       </c>
       <c r="E237">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F237">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G237">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H237">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I237">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J237">
         <v>1</v>
@@ -13048,7 +13048,7 @@
         <v>5</v>
       </c>
       <c r="I238">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J238">
         <v>3</v>
@@ -13130,19 +13130,19 @@
         <v>341</v>
       </c>
       <c r="E240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I240">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J240">
         <v>2</v>
@@ -13224,16 +13224,16 @@
         <v>343</v>
       </c>
       <c r="E242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H242">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I242">
         <v>5</v>
@@ -13298,7 +13298,7 @@
         <v>4</v>
       </c>
       <c r="N243">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O243">
         <v>6</v>
@@ -13318,19 +13318,19 @@
         <v>345</v>
       </c>
       <c r="E244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F244">
         <v>5</v>
       </c>
       <c r="G244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I244">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J244">
         <v>3</v>
@@ -13459,10 +13459,10 @@
         <v>348</v>
       </c>
       <c r="E247">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F247">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G247">
         <v>5</v>
@@ -13600,7 +13600,7 @@
         <v>351</v>
       </c>
       <c r="E250">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F250">
         <v>5</v>
@@ -13662,19 +13662,19 @@
         <v>4</v>
       </c>
       <c r="J251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L251">
         <v>5</v>
       </c>
       <c r="M251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N251">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O251">
         <v>6</v>
@@ -13844,7 +13844,7 @@
         <v>5</v>
       </c>
       <c r="H255">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I255">
         <v>5</v>
@@ -13929,7 +13929,7 @@
         <v>358</v>
       </c>
       <c r="E257">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F257">
         <v>5</v>
@@ -13941,7 +13941,7 @@
         <v>5</v>
       </c>
       <c r="I257">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J257">
         <v>4</v>
@@ -13976,16 +13976,16 @@
         <v>359</v>
       </c>
       <c r="E258">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F258">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G258">
         <v>5</v>
       </c>
       <c r="H258">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I258">
         <v>5</v>
@@ -14026,10 +14026,10 @@
         <v>5</v>
       </c>
       <c r="F259">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G259">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H259">
         <v>4</v>
@@ -14091,13 +14091,13 @@
         <v>4</v>
       </c>
       <c r="L260">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M260">
         <v>5</v>
       </c>
       <c r="N260">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O260">
         <v>6</v>
@@ -14211,19 +14211,19 @@
         <v>364</v>
       </c>
       <c r="E263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F263">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I263">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J263">
         <v>2</v>
@@ -14305,16 +14305,16 @@
         <v>366</v>
       </c>
       <c r="E265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H265">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I265">
         <v>5</v>
@@ -14467,13 +14467,13 @@
         <v>5</v>
       </c>
       <c r="L268">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M268">
         <v>5</v>
       </c>
       <c r="N268">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O268">
         <v>6</v>
@@ -14493,19 +14493,19 @@
         <v>370</v>
       </c>
       <c r="E269">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F269">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G269">
         <v>5</v>
       </c>
       <c r="H269">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I269">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J269">
         <v>2</v>
@@ -14552,7 +14552,7 @@
         <v>5</v>
       </c>
       <c r="I270">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J270">
         <v>3</v>
@@ -14614,7 +14614,7 @@
         <v>4</v>
       </c>
       <c r="N271">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O271">
         <v>6</v>
@@ -14643,7 +14643,7 @@
         <v>5</v>
       </c>
       <c r="H272">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I272">
         <v>5</v>
@@ -14681,7 +14681,7 @@
         <v>374</v>
       </c>
       <c r="E273">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F273">
         <v>5</v>
@@ -14837,16 +14837,16 @@
         <v>4</v>
       </c>
       <c r="J276">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K276">
         <v>5</v>
       </c>
       <c r="L276">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M276">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N276">
         <v>5</v>
@@ -14869,7 +14869,7 @@
         <v>378</v>
       </c>
       <c r="E277">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F277">
         <v>5</v>
@@ -15107,16 +15107,16 @@
         <v>5</v>
       </c>
       <c r="F282">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G282">
         <v>5</v>
       </c>
       <c r="H282">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I282">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J282">
         <v>4</v>
@@ -15178,7 +15178,7 @@
         <v>5</v>
       </c>
       <c r="N283">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O283">
         <v>6</v>
@@ -15351,7 +15351,7 @@
         <v>5</v>
       </c>
       <c r="I287">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J287">
         <v>3</v>
@@ -15386,19 +15386,19 @@
         <v>389</v>
       </c>
       <c r="E288">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F288">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G288">
         <v>5</v>
       </c>
       <c r="H288">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I288">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J288">
         <v>3</v>
@@ -15721,10 +15721,10 @@
         <v>5</v>
       </c>
       <c r="G295">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H295">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I295">
         <v>5</v>
@@ -15856,19 +15856,19 @@
         <v>399</v>
       </c>
       <c r="E298">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H298">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I298">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J298">
         <v>3</v>
@@ -15903,16 +15903,16 @@
         <v>400</v>
       </c>
       <c r="E299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H299">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I299">
         <v>5</v>
@@ -16006,7 +16006,7 @@
         <v>4</v>
       </c>
       <c r="H301">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I301">
         <v>5</v>
@@ -16044,13 +16044,13 @@
         <v>403</v>
       </c>
       <c r="E302">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F302">
         <v>5</v>
       </c>
       <c r="G302">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H302">
         <v>5</v>
@@ -16091,7 +16091,7 @@
         <v>404</v>
       </c>
       <c r="E303">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F303">
         <v>5</v>
@@ -16326,19 +16326,19 @@
         <v>409</v>
       </c>
       <c r="E308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H308">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I308">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J308">
         <v>1</v>
@@ -16467,16 +16467,16 @@
         <v>412</v>
       </c>
       <c r="E311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G311">
         <v>5</v>
       </c>
       <c r="H311">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I311">
         <v>5</v>
@@ -16567,7 +16567,7 @@
         <v>5</v>
       </c>
       <c r="G313">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H313">
         <v>5</v>
@@ -16702,19 +16702,19 @@
         <v>417</v>
       </c>
       <c r="E316">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F316">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G316">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H316">
         <v>5</v>
       </c>
       <c r="I316">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J316">
         <v>2</v>
@@ -16749,16 +16749,16 @@
         <v>418</v>
       </c>
       <c r="E317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H317">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I317">
         <v>5</v>
@@ -16796,7 +16796,7 @@
         <v>419</v>
       </c>
       <c r="E318">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F318">
         <v>5</v>
@@ -16808,7 +16808,7 @@
         <v>5</v>
       </c>
       <c r="I318">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J318">
         <v>1</v>
@@ -16843,16 +16843,16 @@
         <v>420</v>
       </c>
       <c r="E319">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F319">
         <v>5</v>
       </c>
       <c r="G319">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H319">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I319">
         <v>5</v>
@@ -16890,19 +16890,19 @@
         <v>421</v>
       </c>
       <c r="E320">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F320">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G320">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H320">
         <v>5</v>
       </c>
       <c r="I320">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J320">
         <v>2</v>
@@ -17219,7 +17219,7 @@
         <v>428</v>
       </c>
       <c r="E327">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F327">
         <v>5</v>
@@ -17269,7 +17269,7 @@
         <v>4</v>
       </c>
       <c r="F328">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G328">
         <v>5</v>
@@ -17313,19 +17313,19 @@
         <v>430</v>
       </c>
       <c r="E329">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F329">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G329">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H329">
         <v>5</v>
       </c>
       <c r="I329">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J329">
         <v>3</v>
@@ -17454,19 +17454,19 @@
         <v>433</v>
       </c>
       <c r="E332">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F332">
         <v>5</v>
       </c>
       <c r="G332">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H332">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I332">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J332">
         <v>4</v>
@@ -17595,19 +17595,19 @@
         <v>436</v>
       </c>
       <c r="E335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G335">
         <v>4</v>
       </c>
       <c r="H335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I335">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J335">
         <v>1</v>
@@ -17836,7 +17836,7 @@
         <v>5</v>
       </c>
       <c r="G340">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H340">
         <v>5</v>
@@ -17877,7 +17877,7 @@
         <v>442</v>
       </c>
       <c r="E341">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F341">
         <v>4</v>
@@ -17886,7 +17886,7 @@
         <v>4</v>
       </c>
       <c r="H341">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I341">
         <v>5</v>
@@ -17924,19 +17924,19 @@
         <v>443</v>
       </c>
       <c r="E342">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F342">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G342">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H342">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I342">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J342">
         <v>1</v>
@@ -18071,7 +18071,7 @@
         <v>4</v>
       </c>
       <c r="G345">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H345">
         <v>4</v>
@@ -18115,7 +18115,7 @@
         <v>4</v>
       </c>
       <c r="F346">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G346">
         <v>5</v>
@@ -18206,19 +18206,19 @@
         <v>449</v>
       </c>
       <c r="E348">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H348">
         <v>5</v>
       </c>
       <c r="I348">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J348">
         <v>2</v>
@@ -18300,19 +18300,19 @@
         <v>451</v>
       </c>
       <c r="E350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H350">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I350">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J350">
         <v>4</v>
@@ -18347,7 +18347,7 @@
         <v>452</v>
       </c>
       <c r="E351">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F351">
         <v>5</v>
@@ -18356,7 +18356,7 @@
         <v>5</v>
       </c>
       <c r="H351">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I351">
         <v>5</v>
@@ -18400,7 +18400,7 @@
         <v>5</v>
       </c>
       <c r="G352">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H352">
         <v>5</v>
@@ -18488,19 +18488,19 @@
         <v>455</v>
       </c>
       <c r="E354">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F354">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G354">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H354">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I354">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J354">
         <v>4</v>
@@ -18535,19 +18535,19 @@
         <v>456</v>
       </c>
       <c r="E355">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F355">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G355">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H355">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I355">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J355">
         <v>1</v>
@@ -18629,19 +18629,19 @@
         <v>458</v>
       </c>
       <c r="E357">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F357">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G357">
         <v>5</v>
       </c>
       <c r="H357">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I357">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J357">
         <v>2</v>
@@ -18723,7 +18723,7 @@
         <v>460</v>
       </c>
       <c r="E359">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F359">
         <v>5</v>
@@ -18732,10 +18732,10 @@
         <v>5</v>
       </c>
       <c r="H359">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I359">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J359">
         <v>3</v>
@@ -18829,7 +18829,7 @@
         <v>5</v>
       </c>
       <c r="I361">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J361">
         <v>3</v>
@@ -18864,7 +18864,7 @@
         <v>463</v>
       </c>
       <c r="E362">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F362">
         <v>5</v>
@@ -19005,19 +19005,19 @@
         <v>466</v>
       </c>
       <c r="E365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H365">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I365">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J365">
         <v>1</v>
@@ -19052,7 +19052,7 @@
         <v>467</v>
       </c>
       <c r="E366">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F366">
         <v>5</v>
@@ -19108,7 +19108,7 @@
         <v>5</v>
       </c>
       <c r="H367">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I367">
         <v>5</v>
@@ -19146,7 +19146,7 @@
         <v>469</v>
       </c>
       <c r="E368">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F368">
         <v>5</v>
@@ -19199,7 +19199,7 @@
         <v>5</v>
       </c>
       <c r="G369">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H369">
         <v>4</v>
@@ -19340,7 +19340,7 @@
         <v>4</v>
       </c>
       <c r="G372">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H372">
         <v>4</v>
@@ -19475,7 +19475,7 @@
         <v>476</v>
       </c>
       <c r="E375">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F375">
         <v>5</v>
@@ -19522,19 +19522,19 @@
         <v>477</v>
       </c>
       <c r="E376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G376">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I376">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J376">
         <v>4</v>
@@ -19713,7 +19713,7 @@
         <v>5</v>
       </c>
       <c r="F380">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G380">
         <v>5</v>
@@ -19757,13 +19757,13 @@
         <v>482</v>
       </c>
       <c r="E381">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F381">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G381">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H381">
         <v>5</v>
@@ -19804,16 +19804,16 @@
         <v>483</v>
       </c>
       <c r="E382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F382">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G382">
         <v>5</v>
       </c>
       <c r="H382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I382">
         <v>5</v>
@@ -19898,19 +19898,19 @@
         <v>485</v>
       </c>
       <c r="E384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I384">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J384">
         <v>3</v>
@@ -19992,19 +19992,19 @@
         <v>487</v>
       </c>
       <c r="E386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H386">
         <v>5</v>
       </c>
       <c r="I386">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J386">
         <v>3</v>
@@ -20327,10 +20327,10 @@
         <v>5</v>
       </c>
       <c r="G393">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H393">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I393">
         <v>5</v>
@@ -20421,7 +20421,7 @@
         <v>4</v>
       </c>
       <c r="G395">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H395">
         <v>3</v>
@@ -20486,10 +20486,10 @@
         <v>4</v>
       </c>
       <c r="M396">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N396">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O396">
         <v>6</v>
@@ -20512,16 +20512,16 @@
         <v>5</v>
       </c>
       <c r="F397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I397">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J397">
         <v>2</v>
@@ -20650,7 +20650,7 @@
         <v>501</v>
       </c>
       <c r="E400">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F400">
         <v>5</v>
@@ -20659,10 +20659,10 @@
         <v>5</v>
       </c>
       <c r="H400">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I400">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J400">
         <v>4</v>
@@ -20712,7 +20712,7 @@
         <v>4</v>
       </c>
       <c r="J401">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K401">
         <v>5</v>

</xml_diff>

<commit_message>
fix(corr): BE-ME from -0.43*** to -0.08 (ns) — benign and malicious envy are conceptually distinct reactions, should be weakly correlated or near zero (not strong negative). rebuild_340.py pair_corr -0.417→-0.05; full rebuild+R+overlay+validate. 219/219+10/10.
</commit_message>
<xml_diff>
--- a/data/T2_cleaned.xlsx
+++ b/data/T2_cleaned.xlsx
@@ -1962,19 +1962,19 @@
         <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -2062,7 +2062,7 @@
         <v>3</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4">
         <v>2</v>
@@ -2109,7 +2109,7 @@
         <v>2</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -2200,13 +2200,13 @@
         <v>2</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -2250,10 +2250,10 @@
         <v>3</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8">
         <v>3</v>
@@ -2347,10 +2347,10 @@
         <v>4</v>
       </c>
       <c r="M10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -2526,16 +2526,16 @@
         <v>6</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K14">
         <v>3</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14">
         <v>3</v>
@@ -2573,19 +2573,19 @@
         <v>5</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15">
         <v>6</v>
@@ -2620,19 +2620,19 @@
         <v>5</v>
       </c>
       <c r="J16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16">
         <v>1</v>
       </c>
       <c r="N16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16">
         <v>6</v>
@@ -2667,19 +2667,19 @@
         <v>5</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17">
         <v>2</v>
       </c>
       <c r="M17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -2761,16 +2761,16 @@
         <v>5</v>
       </c>
       <c r="J19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19">
         <v>2</v>
@@ -2808,19 +2808,19 @@
         <v>4</v>
       </c>
       <c r="J20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2858,7 +2858,7 @@
         <v>4</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L21">
         <v>4</v>
@@ -2902,7 +2902,7 @@
         <v>5</v>
       </c>
       <c r="J22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K22">
         <v>4</v>
@@ -2911,7 +2911,7 @@
         <v>5</v>
       </c>
       <c r="M22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N22">
         <v>4</v>
@@ -2949,19 +2949,19 @@
         <v>3</v>
       </c>
       <c r="J23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L23">
         <v>4</v>
       </c>
       <c r="M23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23">
         <v>6</v>
@@ -3093,7 +3093,7 @@
         <v>4</v>
       </c>
       <c r="K26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L26">
         <v>3</v>
@@ -3187,13 +3187,13 @@
         <v>3</v>
       </c>
       <c r="K28">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L28">
         <v>3</v>
       </c>
       <c r="M28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N28">
         <v>2</v>
@@ -3231,16 +3231,16 @@
         <v>4</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N29">
         <v>5</v>
@@ -3325,16 +3325,16 @@
         <v>3</v>
       </c>
       <c r="J31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L31">
         <v>4</v>
       </c>
       <c r="M31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N31">
         <v>4</v>
@@ -3431,7 +3431,7 @@
         <v>2</v>
       </c>
       <c r="N33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -3469,10 +3469,10 @@
         <v>4</v>
       </c>
       <c r="K34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M34">
         <v>4</v>
@@ -3513,7 +3513,7 @@
         <v>5</v>
       </c>
       <c r="J35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K35">
         <v>3</v>
@@ -3522,10 +3522,10 @@
         <v>2</v>
       </c>
       <c r="M35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O35">
         <v>6</v>
@@ -3563,16 +3563,16 @@
         <v>4</v>
       </c>
       <c r="K36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -3607,19 +3607,19 @@
         <v>3</v>
       </c>
       <c r="J37">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N37">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -3657,7 +3657,7 @@
         <v>2</v>
       </c>
       <c r="K38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L38">
         <v>1</v>
@@ -3701,19 +3701,19 @@
         <v>2</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3845,13 +3845,13 @@
         <v>3</v>
       </c>
       <c r="K42">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N42">
         <v>2</v>
@@ -3989,7 +3989,7 @@
         <v>5</v>
       </c>
       <c r="L45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M45">
         <v>4</v>
@@ -4030,16 +4030,16 @@
         <v>4</v>
       </c>
       <c r="J46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N46">
         <v>4</v>
@@ -4077,19 +4077,19 @@
         <v>6</v>
       </c>
       <c r="J47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O47">
         <v>6</v>
@@ -4124,19 +4124,19 @@
         <v>7</v>
       </c>
       <c r="J48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K48">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M48">
         <v>3</v>
       </c>
       <c r="N48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O48">
         <v>6</v>
@@ -4174,7 +4174,7 @@
         <v>1</v>
       </c>
       <c r="K49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49">
         <v>1</v>
@@ -4218,19 +4218,19 @@
         <v>6</v>
       </c>
       <c r="J50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4315,13 +4315,13 @@
         <v>1</v>
       </c>
       <c r="K52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52">
         <v>1</v>
@@ -4359,16 +4359,16 @@
         <v>7</v>
       </c>
       <c r="J53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L53">
         <v>4</v>
       </c>
       <c r="M53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N53">
         <v>2</v>
@@ -4409,16 +4409,16 @@
         <v>2</v>
       </c>
       <c r="K54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4506,7 +4506,7 @@
         <v>1</v>
       </c>
       <c r="L56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M56">
         <v>1</v>
@@ -4556,10 +4556,10 @@
         <v>3</v>
       </c>
       <c r="M57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4691,7 +4691,7 @@
         <v>3</v>
       </c>
       <c r="K60">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L60">
         <v>3</v>
@@ -4876,7 +4876,7 @@
         <v>3</v>
       </c>
       <c r="J64">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K64">
         <v>5</v>
@@ -4923,19 +4923,19 @@
         <v>3</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L65">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N65">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -4970,19 +4970,19 @@
         <v>7</v>
       </c>
       <c r="J66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5020,7 +5020,7 @@
         <v>4</v>
       </c>
       <c r="K67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L67">
         <v>3</v>
@@ -5158,19 +5158,19 @@
         <v>2</v>
       </c>
       <c r="J70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O70">
         <v>6</v>
@@ -5205,16 +5205,16 @@
         <v>3</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N71">
         <v>3</v>
@@ -5252,19 +5252,19 @@
         <v>4</v>
       </c>
       <c r="J72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K72">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N72">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O72">
         <v>6</v>
@@ -5299,19 +5299,19 @@
         <v>7</v>
       </c>
       <c r="J73">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5346,19 +5346,19 @@
         <v>7</v>
       </c>
       <c r="J74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5396,7 +5396,7 @@
         <v>1</v>
       </c>
       <c r="K75">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L75">
         <v>4</v>
@@ -5443,10 +5443,10 @@
         <v>2</v>
       </c>
       <c r="K76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M76">
         <v>1</v>
@@ -5487,19 +5487,19 @@
         <v>3</v>
       </c>
       <c r="J77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5546,7 +5546,7 @@
         <v>1</v>
       </c>
       <c r="N78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5581,7 +5581,7 @@
         <v>5</v>
       </c>
       <c r="J79">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K79">
         <v>4</v>
@@ -5593,7 +5593,7 @@
         <v>4</v>
       </c>
       <c r="N79">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -5628,19 +5628,19 @@
         <v>7</v>
       </c>
       <c r="J80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O80">
         <v>6</v>
@@ -5772,7 +5772,7 @@
         <v>3</v>
       </c>
       <c r="K83">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L83">
         <v>3</v>
@@ -5816,19 +5816,19 @@
         <v>4</v>
       </c>
       <c r="J84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K84">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O84">
         <v>6</v>
@@ -5863,19 +5863,19 @@
         <v>2</v>
       </c>
       <c r="J85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K85">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O85">
         <v>6</v>
@@ -5910,19 +5910,19 @@
         <v>7</v>
       </c>
       <c r="J86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L86">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M86">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N86">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O86">
         <v>6</v>
@@ -6007,13 +6007,13 @@
         <v>2</v>
       </c>
       <c r="K88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L88">
         <v>3</v>
       </c>
       <c r="M88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N88">
         <v>2</v>
@@ -6051,19 +6051,19 @@
         <v>4</v>
       </c>
       <c r="J89">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M89">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O89">
         <v>6</v>
@@ -6098,19 +6098,19 @@
         <v>7</v>
       </c>
       <c r="J90">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L90">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M90">
         <v>3</v>
       </c>
       <c r="N90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O90">
         <v>6</v>
@@ -6145,19 +6145,19 @@
         <v>7</v>
       </c>
       <c r="J91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K91">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L91">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M91">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O91">
         <v>6</v>
@@ -6239,19 +6239,19 @@
         <v>4</v>
       </c>
       <c r="J93">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K93">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L93">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M93">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N93">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O93">
         <v>6</v>
@@ -6286,19 +6286,19 @@
         <v>5</v>
       </c>
       <c r="J94">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K94">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L94">
         <v>2</v>
       </c>
       <c r="M94">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N94">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O94">
         <v>6</v>
@@ -6383,16 +6383,16 @@
         <v>1</v>
       </c>
       <c r="K96">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M96">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O96">
         <v>6</v>
@@ -6521,16 +6521,16 @@
         <v>3</v>
       </c>
       <c r="J99">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K99">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L99">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M99">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N99">
         <v>3</v>
@@ -6574,7 +6574,7 @@
         <v>3</v>
       </c>
       <c r="L100">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M100">
         <v>6</v>
@@ -6615,19 +6615,19 @@
         <v>6</v>
       </c>
       <c r="J101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K101">
         <v>3</v>
       </c>
       <c r="L101">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O101">
         <v>6</v>
@@ -6712,16 +6712,16 @@
         <v>4</v>
       </c>
       <c r="K103">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L103">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M103">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N103">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O103">
         <v>6</v>
@@ -6756,19 +6756,19 @@
         <v>6</v>
       </c>
       <c r="J104">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K104">
         <v>1</v>
       </c>
       <c r="L104">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M104">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N104">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O104">
         <v>6</v>
@@ -6803,16 +6803,16 @@
         <v>7</v>
       </c>
       <c r="J105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K105">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M105">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N105">
         <v>1</v>
@@ -6897,7 +6897,7 @@
         <v>5</v>
       </c>
       <c r="J107">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K107">
         <v>3</v>
@@ -7000,7 +7000,7 @@
         <v>1</v>
       </c>
       <c r="M109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N109">
         <v>2</v>
@@ -7038,19 +7038,19 @@
         <v>1</v>
       </c>
       <c r="J110">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K110">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L110">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M110">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N110">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O110">
         <v>6</v>
@@ -7132,19 +7132,19 @@
         <v>4</v>
       </c>
       <c r="J112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N112">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O112">
         <v>6</v>
@@ -7179,13 +7179,13 @@
         <v>4</v>
       </c>
       <c r="J113">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K113">
         <v>1</v>
       </c>
       <c r="L113">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M113">
         <v>1</v>
@@ -7273,19 +7273,19 @@
         <v>3</v>
       </c>
       <c r="J115">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K115">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L115">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M115">
         <v>4</v>
       </c>
       <c r="N115">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O115">
         <v>6</v>
@@ -7320,19 +7320,19 @@
         <v>3</v>
       </c>
       <c r="J116">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K116">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L116">
         <v>3</v>
       </c>
       <c r="M116">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N116">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O116">
         <v>6</v>
@@ -7367,7 +7367,7 @@
         <v>4</v>
       </c>
       <c r="J117">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K117">
         <v>3</v>
@@ -7379,7 +7379,7 @@
         <v>4</v>
       </c>
       <c r="N117">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O117">
         <v>6</v>
@@ -7558,13 +7558,13 @@
         <v>3</v>
       </c>
       <c r="K121">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L121">
         <v>3</v>
       </c>
       <c r="M121">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N121">
         <v>4</v>
@@ -7602,13 +7602,13 @@
         <v>6</v>
       </c>
       <c r="J122">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K122">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L122">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M122">
         <v>5</v>
@@ -7802,7 +7802,7 @@
         <v>2</v>
       </c>
       <c r="N126">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O126">
         <v>6</v>
@@ -7849,7 +7849,7 @@
         <v>5</v>
       </c>
       <c r="N127">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O127">
         <v>6</v>
@@ -7931,13 +7931,13 @@
         <v>4</v>
       </c>
       <c r="J129">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K129">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M129">
         <v>7</v>
@@ -7978,19 +7978,19 @@
         <v>7</v>
       </c>
       <c r="J130">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K130">
         <v>3</v>
       </c>
       <c r="L130">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M130">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N130">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O130">
         <v>6</v>
@@ -8072,19 +8072,19 @@
         <v>5</v>
       </c>
       <c r="J132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M132">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O132">
         <v>6</v>
@@ -8119,19 +8119,19 @@
         <v>3</v>
       </c>
       <c r="J133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N133">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O133">
         <v>6</v>
@@ -8166,19 +8166,19 @@
         <v>2</v>
       </c>
       <c r="J134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O134">
         <v>6</v>
@@ -8260,19 +8260,19 @@
         <v>6</v>
       </c>
       <c r="J136">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K136">
         <v>3</v>
       </c>
       <c r="L136">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M136">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N136">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O136">
         <v>6</v>
@@ -8307,19 +8307,19 @@
         <v>3</v>
       </c>
       <c r="J137">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K137">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L137">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M137">
         <v>2</v>
       </c>
       <c r="N137">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O137">
         <v>6</v>
@@ -8354,19 +8354,19 @@
         <v>4</v>
       </c>
       <c r="J138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K138">
         <v>3</v>
       </c>
       <c r="L138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M138">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O138">
         <v>6</v>
@@ -8404,7 +8404,7 @@
         <v>4</v>
       </c>
       <c r="K139">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L139">
         <v>3</v>
@@ -8448,19 +8448,19 @@
         <v>5</v>
       </c>
       <c r="J140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K140">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L140">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O140">
         <v>6</v>
@@ -8592,7 +8592,7 @@
         <v>4</v>
       </c>
       <c r="K143">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L143">
         <v>3</v>
@@ -8636,7 +8636,7 @@
         <v>5</v>
       </c>
       <c r="J144">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K144">
         <v>5</v>
@@ -8739,7 +8739,7 @@
         <v>3</v>
       </c>
       <c r="M146">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N146">
         <v>4</v>
@@ -8777,19 +8777,19 @@
         <v>6</v>
       </c>
       <c r="J147">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K147">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L147">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M147">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N147">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O147">
         <v>6</v>
@@ -8830,7 +8830,7 @@
         <v>3</v>
       </c>
       <c r="L148">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M148">
         <v>4</v>
@@ -8883,7 +8883,7 @@
         <v>4</v>
       </c>
       <c r="N149">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O149">
         <v>6</v>
@@ -8921,16 +8921,16 @@
         <v>6</v>
       </c>
       <c r="K150">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L150">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M150">
         <v>4</v>
       </c>
       <c r="N150">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O150">
         <v>6</v>
@@ -8968,16 +8968,16 @@
         <v>1</v>
       </c>
       <c r="K151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O151">
         <v>6</v>
@@ -9109,10 +9109,10 @@
         <v>1</v>
       </c>
       <c r="K154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M154">
         <v>1</v>
@@ -9162,7 +9162,7 @@
         <v>4</v>
       </c>
       <c r="M155">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N155">
         <v>2</v>
@@ -9200,7 +9200,7 @@
         <v>6</v>
       </c>
       <c r="J156">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K156">
         <v>3</v>
@@ -9209,7 +9209,7 @@
         <v>3</v>
       </c>
       <c r="M156">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N156">
         <v>4</v>
@@ -9247,19 +9247,19 @@
         <v>7</v>
       </c>
       <c r="J157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K157">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M157">
         <v>3</v>
       </c>
       <c r="N157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O157">
         <v>6</v>
@@ -9297,16 +9297,16 @@
         <v>4</v>
       </c>
       <c r="K158">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L158">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M158">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N158">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O158">
         <v>6</v>
@@ -9400,7 +9400,7 @@
         <v>3</v>
       </c>
       <c r="N160">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O160">
         <v>6</v>
@@ -9435,19 +9435,19 @@
         <v>3</v>
       </c>
       <c r="J161">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K161">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L161">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M161">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N161">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O161">
         <v>6</v>
@@ -9541,7 +9541,7 @@
         <v>1</v>
       </c>
       <c r="N163">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O163">
         <v>6</v>
@@ -9579,7 +9579,7 @@
         <v>3</v>
       </c>
       <c r="K164">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L164">
         <v>3</v>
@@ -9673,13 +9673,13 @@
         <v>3</v>
       </c>
       <c r="K166">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L166">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M166">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N166">
         <v>3</v>
@@ -9764,10 +9764,10 @@
         <v>5</v>
       </c>
       <c r="J168">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K168">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L168">
         <v>3</v>
@@ -9858,19 +9858,19 @@
         <v>4</v>
       </c>
       <c r="J170">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K170">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L170">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M170">
         <v>4</v>
       </c>
       <c r="N170">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O170">
         <v>6</v>
@@ -9905,19 +9905,19 @@
         <v>5</v>
       </c>
       <c r="J171">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K171">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L171">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M171">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N171">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O171">
         <v>6</v>
@@ -9952,19 +9952,19 @@
         <v>6</v>
       </c>
       <c r="J172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K172">
         <v>3</v>
       </c>
       <c r="L172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M172">
         <v>4</v>
       </c>
       <c r="N172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O172">
         <v>6</v>
@@ -9999,19 +9999,19 @@
         <v>5</v>
       </c>
       <c r="J173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K173">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M173">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N173">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O173">
         <v>6</v>
@@ -10055,7 +10055,7 @@
         <v>3</v>
       </c>
       <c r="M174">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N174">
         <v>2</v>
@@ -10140,7 +10140,7 @@
         <v>6</v>
       </c>
       <c r="J176">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K176">
         <v>1</v>
@@ -10293,7 +10293,7 @@
         <v>3</v>
       </c>
       <c r="N179">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O179">
         <v>6</v>
@@ -10331,7 +10331,7 @@
         <v>3</v>
       </c>
       <c r="K180">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L180">
         <v>4</v>
@@ -10469,10 +10469,10 @@
         <v>5</v>
       </c>
       <c r="J183">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K183">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L183">
         <v>1</v>
@@ -10516,19 +10516,19 @@
         <v>5</v>
       </c>
       <c r="J184">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K184">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L184">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M184">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N184">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O184">
         <v>6</v>
@@ -10569,10 +10569,10 @@
         <v>4</v>
       </c>
       <c r="L185">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M185">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N185">
         <v>3</v>
@@ -10619,10 +10619,10 @@
         <v>5</v>
       </c>
       <c r="M186">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N186">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O186">
         <v>6</v>
@@ -10657,16 +10657,16 @@
         <v>4</v>
       </c>
       <c r="J187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K187">
         <v>3</v>
       </c>
       <c r="L187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N187">
         <v>4</v>
@@ -10986,19 +10986,19 @@
         <v>7</v>
       </c>
       <c r="J194">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K194">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L194">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M194">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N194">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O194">
         <v>6</v>
@@ -11036,10 +11036,10 @@
         <v>4</v>
       </c>
       <c r="K195">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L195">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M195">
         <v>5</v>
@@ -11080,19 +11080,19 @@
         <v>1</v>
       </c>
       <c r="J196">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K196">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L196">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M196">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N196">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O196">
         <v>6</v>
@@ -11127,10 +11127,10 @@
         <v>4</v>
       </c>
       <c r="J197">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K197">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L197">
         <v>4</v>
@@ -11174,7 +11174,7 @@
         <v>3</v>
       </c>
       <c r="J198">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K198">
         <v>5</v>
@@ -11268,16 +11268,16 @@
         <v>6</v>
       </c>
       <c r="J200">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K200">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L200">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M200">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N200">
         <v>4</v>
@@ -11315,19 +11315,19 @@
         <v>3</v>
       </c>
       <c r="J201">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K201">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L201">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M201">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N201">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O201">
         <v>6</v>
@@ -11362,19 +11362,19 @@
         <v>2</v>
       </c>
       <c r="J202">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K202">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L202">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M202">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N202">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O202">
         <v>6</v>
@@ -11409,7 +11409,7 @@
         <v>2</v>
       </c>
       <c r="J203">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K203">
         <v>2</v>
@@ -11456,19 +11456,19 @@
         <v>4</v>
       </c>
       <c r="J204">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K204">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L204">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M204">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N204">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O204">
         <v>6</v>
@@ -11512,10 +11512,10 @@
         <v>5</v>
       </c>
       <c r="M205">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N205">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O205">
         <v>6</v>
@@ -11550,19 +11550,19 @@
         <v>4</v>
       </c>
       <c r="J206">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K206">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L206">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M206">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N206">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O206">
         <v>6</v>
@@ -11600,7 +11600,7 @@
         <v>4</v>
       </c>
       <c r="K207">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L207">
         <v>4</v>
@@ -11644,10 +11644,10 @@
         <v>4</v>
       </c>
       <c r="J208">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K208">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L208">
         <v>2</v>
@@ -11656,7 +11656,7 @@
         <v>2</v>
       </c>
       <c r="N208">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O208">
         <v>6</v>
@@ -11700,7 +11700,7 @@
         <v>3</v>
       </c>
       <c r="M209">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N209">
         <v>3</v>
@@ -11785,19 +11785,19 @@
         <v>1</v>
       </c>
       <c r="J211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O211">
         <v>6</v>
@@ -11835,16 +11835,16 @@
         <v>4</v>
       </c>
       <c r="K212">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L212">
         <v>4</v>
       </c>
       <c r="M212">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N212">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O212">
         <v>6</v>
@@ -11926,7 +11926,7 @@
         <v>5</v>
       </c>
       <c r="J214">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K214">
         <v>2</v>
@@ -11976,7 +11976,7 @@
         <v>2</v>
       </c>
       <c r="K215">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L215">
         <v>1</v>
@@ -11985,7 +11985,7 @@
         <v>4</v>
       </c>
       <c r="N215">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O215">
         <v>6</v>
@@ -12076,10 +12076,10 @@
         <v>3</v>
       </c>
       <c r="M217">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N217">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O217">
         <v>6</v>
@@ -12161,16 +12161,16 @@
         <v>3</v>
       </c>
       <c r="J219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N219">
         <v>1</v>
@@ -12264,7 +12264,7 @@
         <v>2</v>
       </c>
       <c r="M221">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N221">
         <v>1</v>
@@ -12349,19 +12349,19 @@
         <v>4</v>
       </c>
       <c r="J223">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K223">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L223">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M223">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N223">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O223">
         <v>6</v>
@@ -12443,10 +12443,10 @@
         <v>3</v>
       </c>
       <c r="J225">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K225">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L225">
         <v>2</v>
@@ -12455,7 +12455,7 @@
         <v>2</v>
       </c>
       <c r="N225">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O225">
         <v>6</v>
@@ -12502,7 +12502,7 @@
         <v>1</v>
       </c>
       <c r="N226">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O226">
         <v>6</v>
@@ -12584,10 +12584,10 @@
         <v>6</v>
       </c>
       <c r="J228">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K228">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L228">
         <v>2</v>
@@ -12596,7 +12596,7 @@
         <v>2</v>
       </c>
       <c r="N228">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O228">
         <v>6</v>
@@ -12637,7 +12637,7 @@
         <v>2</v>
       </c>
       <c r="L229">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M229">
         <v>1</v>
@@ -12731,7 +12731,7 @@
         <v>2</v>
       </c>
       <c r="L231">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M231">
         <v>1</v>
@@ -12866,19 +12866,19 @@
         <v>5</v>
       </c>
       <c r="J234">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K234">
         <v>3</v>
       </c>
       <c r="L234">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M234">
         <v>3</v>
       </c>
       <c r="N234">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O234">
         <v>6</v>
@@ -12913,16 +12913,16 @@
         <v>5</v>
       </c>
       <c r="J235">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K235">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L235">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M235">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N235">
         <v>3</v>
@@ -12960,19 +12960,19 @@
         <v>5</v>
       </c>
       <c r="J236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M236">
         <v>3</v>
       </c>
       <c r="N236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O236">
         <v>6</v>
@@ -13007,19 +13007,19 @@
         <v>6</v>
       </c>
       <c r="J237">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K237">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L237">
         <v>4</v>
       </c>
       <c r="M237">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N237">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O237">
         <v>6</v>
@@ -13054,10 +13054,10 @@
         <v>6</v>
       </c>
       <c r="J238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L238">
         <v>3</v>
@@ -13066,7 +13066,7 @@
         <v>1</v>
       </c>
       <c r="N238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O238">
         <v>6</v>
@@ -13107,7 +13107,7 @@
         <v>2</v>
       </c>
       <c r="L239">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M239">
         <v>2</v>
@@ -13160,7 +13160,7 @@
         <v>5</v>
       </c>
       <c r="N240">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O240">
         <v>6</v>
@@ -13195,19 +13195,19 @@
         <v>4</v>
       </c>
       <c r="J241">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K241">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L241">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M241">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N241">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O241">
         <v>6</v>
@@ -13242,19 +13242,19 @@
         <v>5</v>
       </c>
       <c r="J242">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N242">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O242">
         <v>6</v>
@@ -13295,7 +13295,7 @@
         <v>3</v>
       </c>
       <c r="L243">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M243">
         <v>2</v>
@@ -13436,7 +13436,7 @@
         <v>1</v>
       </c>
       <c r="L246">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M246">
         <v>1</v>
@@ -13536,7 +13536,7 @@
         <v>1</v>
       </c>
       <c r="N248">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O248">
         <v>6</v>
@@ -13580,7 +13580,7 @@
         <v>1</v>
       </c>
       <c r="M249">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N249">
         <v>2</v>
@@ -13624,10 +13624,10 @@
         <v>5</v>
       </c>
       <c r="L250">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M250">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N250">
         <v>5</v>
@@ -13859,7 +13859,7 @@
         <v>4</v>
       </c>
       <c r="L255">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M255">
         <v>4</v>
@@ -13994,19 +13994,19 @@
         <v>4</v>
       </c>
       <c r="J258">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K258">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L258">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M258">
         <v>2</v>
       </c>
       <c r="N258">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O258">
         <v>6</v>
@@ -14088,19 +14088,19 @@
         <v>4</v>
       </c>
       <c r="J260">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K260">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L260">
         <v>5</v>
       </c>
       <c r="M260">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N260">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O260">
         <v>6</v>
@@ -14182,13 +14182,13 @@
         <v>1</v>
       </c>
       <c r="J262">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K262">
         <v>3</v>
       </c>
       <c r="L262">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M262">
         <v>4</v>
@@ -14232,16 +14232,16 @@
         <v>4</v>
       </c>
       <c r="K263">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L263">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M263">
         <v>4</v>
       </c>
       <c r="N263">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O263">
         <v>6</v>
@@ -14376,10 +14376,10 @@
         <v>1</v>
       </c>
       <c r="L266">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M266">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N266">
         <v>1</v>
@@ -14417,16 +14417,16 @@
         <v>4</v>
       </c>
       <c r="J267">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K267">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L267">
         <v>2</v>
       </c>
       <c r="M267">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N267">
         <v>3</v>
@@ -14470,7 +14470,7 @@
         <v>5</v>
       </c>
       <c r="L268">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M268">
         <v>6</v>
@@ -14511,19 +14511,19 @@
         <v>7</v>
       </c>
       <c r="J269">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K269">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L269">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M269">
         <v>3</v>
       </c>
       <c r="N269">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O269">
         <v>6</v>
@@ -14558,7 +14558,7 @@
         <v>7</v>
       </c>
       <c r="J270">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K270">
         <v>3</v>
@@ -14614,7 +14614,7 @@
         <v>1</v>
       </c>
       <c r="M271">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N271">
         <v>1</v>
@@ -14708,7 +14708,7 @@
         <v>2</v>
       </c>
       <c r="M273">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N273">
         <v>4</v>
@@ -14746,13 +14746,13 @@
         <v>3</v>
       </c>
       <c r="J274">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K274">
         <v>2</v>
       </c>
       <c r="L274">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M274">
         <v>2</v>
@@ -14840,16 +14840,16 @@
         <v>3</v>
       </c>
       <c r="J276">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K276">
         <v>4</v>
       </c>
       <c r="L276">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M276">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N276">
         <v>6</v>
@@ -14896,10 +14896,10 @@
         <v>4</v>
       </c>
       <c r="M277">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N277">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O277">
         <v>6</v>
@@ -14981,19 +14981,19 @@
         <v>6</v>
       </c>
       <c r="J279">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K279">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L279">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M279">
         <v>4</v>
       </c>
       <c r="N279">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O279">
         <v>6</v>
@@ -15028,7 +15028,7 @@
         <v>3</v>
       </c>
       <c r="J280">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K280">
         <v>1</v>
@@ -15037,10 +15037,10 @@
         <v>2</v>
       </c>
       <c r="M280">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N280">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O280">
         <v>6</v>
@@ -15078,7 +15078,7 @@
         <v>4</v>
       </c>
       <c r="K281">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L281">
         <v>3</v>
@@ -15134,7 +15134,7 @@
         <v>3</v>
       </c>
       <c r="N282">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O282">
         <v>6</v>
@@ -15169,7 +15169,7 @@
         <v>4</v>
       </c>
       <c r="J283">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K283">
         <v>2</v>
@@ -15216,19 +15216,19 @@
         <v>7</v>
       </c>
       <c r="J284">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K284">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L284">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M284">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N284">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O284">
         <v>6</v>
@@ -15313,7 +15313,7 @@
         <v>6</v>
       </c>
       <c r="K286">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L286">
         <v>6</v>
@@ -15366,7 +15366,7 @@
         <v>1</v>
       </c>
       <c r="M287">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N287">
         <v>1</v>
@@ -15451,7 +15451,7 @@
         <v>3</v>
       </c>
       <c r="J289">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K289">
         <v>1</v>
@@ -15504,13 +15504,13 @@
         <v>4</v>
       </c>
       <c r="L290">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M290">
         <v>6</v>
       </c>
       <c r="N290">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O290">
         <v>6</v>
@@ -15545,19 +15545,19 @@
         <v>2</v>
       </c>
       <c r="J291">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K291">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L291">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M291">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N291">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O291">
         <v>6</v>
@@ -15595,13 +15595,13 @@
         <v>3</v>
       </c>
       <c r="K292">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L292">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M292">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N292">
         <v>2</v>
@@ -15639,19 +15639,19 @@
         <v>5</v>
       </c>
       <c r="J293">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K293">
         <v>4</v>
       </c>
       <c r="L293">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M293">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N293">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O293">
         <v>6</v>
@@ -15780,19 +15780,19 @@
         <v>3</v>
       </c>
       <c r="J296">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K296">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L296">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M296">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N296">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O296">
         <v>6</v>
@@ -15830,7 +15830,7 @@
         <v>2</v>
       </c>
       <c r="K297">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L297">
         <v>2</v>
@@ -15839,7 +15839,7 @@
         <v>3</v>
       </c>
       <c r="N297">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O297">
         <v>6</v>
@@ -15874,19 +15874,19 @@
         <v>3</v>
       </c>
       <c r="J298">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K298">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L298">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M298">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N298">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O298">
         <v>6</v>
@@ -15924,16 +15924,16 @@
         <v>4</v>
       </c>
       <c r="K299">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L299">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M299">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N299">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O299">
         <v>6</v>
@@ -15968,19 +15968,19 @@
         <v>5</v>
       </c>
       <c r="J300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L300">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O300">
         <v>6</v>
@@ -16015,19 +16015,19 @@
         <v>7</v>
       </c>
       <c r="J301">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K301">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L301">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M301">
         <v>2</v>
       </c>
       <c r="N301">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O301">
         <v>6</v>
@@ -16112,16 +16112,16 @@
         <v>2</v>
       </c>
       <c r="K303">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L303">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M303">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N303">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O303">
         <v>6</v>
@@ -16156,19 +16156,19 @@
         <v>3</v>
       </c>
       <c r="J304">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K304">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L304">
         <v>4</v>
       </c>
       <c r="M304">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N304">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O304">
         <v>6</v>
@@ -16203,19 +16203,19 @@
         <v>6</v>
       </c>
       <c r="J305">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K305">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L305">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M305">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N305">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O305">
         <v>6</v>
@@ -16250,19 +16250,19 @@
         <v>6</v>
       </c>
       <c r="J306">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K306">
         <v>3</v>
       </c>
       <c r="L306">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M306">
         <v>4</v>
       </c>
       <c r="N306">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O306">
         <v>6</v>
@@ -16300,16 +16300,16 @@
         <v>2</v>
       </c>
       <c r="K307">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L307">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M307">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N307">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O307">
         <v>6</v>
@@ -16347,7 +16347,7 @@
         <v>3</v>
       </c>
       <c r="K308">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L308">
         <v>3</v>
@@ -16391,19 +16391,19 @@
         <v>4</v>
       </c>
       <c r="J309">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K309">
         <v>3</v>
       </c>
       <c r="L309">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M309">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N309">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O309">
         <v>6</v>
@@ -16485,7 +16485,7 @@
         <v>5</v>
       </c>
       <c r="J311">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K311">
         <v>4</v>
@@ -16582,13 +16582,13 @@
         <v>2</v>
       </c>
       <c r="K313">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L313">
         <v>3</v>
       </c>
       <c r="M313">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N313">
         <v>2</v>
@@ -16635,10 +16635,10 @@
         <v>4</v>
       </c>
       <c r="M314">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N314">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O314">
         <v>6</v>
@@ -16673,13 +16673,13 @@
         <v>6</v>
       </c>
       <c r="J315">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K315">
         <v>4</v>
       </c>
       <c r="L315">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M315">
         <v>3</v>
@@ -16720,19 +16720,19 @@
         <v>6</v>
       </c>
       <c r="J316">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M316">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O316">
         <v>6</v>
@@ -16814,19 +16814,19 @@
         <v>6</v>
       </c>
       <c r="J318">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K318">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L318">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M318">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N318">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O318">
         <v>6</v>
@@ -16864,13 +16864,13 @@
         <v>4</v>
       </c>
       <c r="K319">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L319">
         <v>4</v>
       </c>
       <c r="M319">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N319">
         <v>4</v>
@@ -16911,16 +16911,16 @@
         <v>1</v>
       </c>
       <c r="K320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M320">
         <v>1</v>
       </c>
       <c r="N320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O320">
         <v>6</v>
@@ -17143,19 +17143,19 @@
         <v>3</v>
       </c>
       <c r="J325">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K325">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L325">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M325">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N325">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O325">
         <v>6</v>
@@ -17237,19 +17237,19 @@
         <v>4</v>
       </c>
       <c r="J327">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K327">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L327">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M327">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N327">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O327">
         <v>6</v>
@@ -17284,7 +17284,7 @@
         <v>6</v>
       </c>
       <c r="J328">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K328">
         <v>2</v>
@@ -17296,7 +17296,7 @@
         <v>5</v>
       </c>
       <c r="N328">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O328">
         <v>6</v>
@@ -17331,16 +17331,16 @@
         <v>4</v>
       </c>
       <c r="J329">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K329">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L329">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M329">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N329">
         <v>1</v>
@@ -17384,13 +17384,13 @@
         <v>2</v>
       </c>
       <c r="L330">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M330">
         <v>3</v>
       </c>
       <c r="N330">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O330">
         <v>6</v>
@@ -17425,19 +17425,19 @@
         <v>7</v>
       </c>
       <c r="J331">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K331">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L331">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M331">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N331">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O331">
         <v>6</v>
@@ -17472,16 +17472,16 @@
         <v>4</v>
       </c>
       <c r="J332">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K332">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L332">
         <v>4</v>
       </c>
       <c r="M332">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N332">
         <v>4</v>
@@ -17519,19 +17519,19 @@
         <v>6</v>
       </c>
       <c r="J333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L333">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O333">
         <v>6</v>
@@ -17566,7 +17566,7 @@
         <v>5</v>
       </c>
       <c r="J334">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K334">
         <v>2</v>
@@ -17660,19 +17660,19 @@
         <v>6</v>
       </c>
       <c r="J336">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K336">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L336">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M336">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N336">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O336">
         <v>6</v>
@@ -17707,19 +17707,19 @@
         <v>3</v>
       </c>
       <c r="J337">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K337">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L337">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M337">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N337">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O337">
         <v>6</v>
@@ -17804,7 +17804,7 @@
         <v>3</v>
       </c>
       <c r="K339">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L339">
         <v>4</v>
@@ -17895,19 +17895,19 @@
         <v>5</v>
       </c>
       <c r="J341">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K341">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L341">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M341">
         <v>2</v>
       </c>
       <c r="N341">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O341">
         <v>6</v>
@@ -18036,19 +18036,19 @@
         <v>3</v>
       </c>
       <c r="J344">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K344">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L344">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M344">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N344">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O344">
         <v>6</v>
@@ -18083,10 +18083,10 @@
         <v>5</v>
       </c>
       <c r="J345">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K345">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L345">
         <v>5</v>
@@ -18139,7 +18139,7 @@
         <v>4</v>
       </c>
       <c r="M346">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N346">
         <v>4</v>
@@ -18180,13 +18180,13 @@
         <v>2</v>
       </c>
       <c r="K347">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L347">
         <v>2</v>
       </c>
       <c r="M347">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N347">
         <v>1</v>
@@ -18283,7 +18283,7 @@
         <v>4</v>
       </c>
       <c r="N349">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O349">
         <v>6</v>
@@ -18327,7 +18327,7 @@
         <v>4</v>
       </c>
       <c r="M350">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N350">
         <v>4</v>
@@ -18412,19 +18412,19 @@
         <v>7</v>
       </c>
       <c r="J352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K352">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N352">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O352">
         <v>6</v>
@@ -18459,13 +18459,13 @@
         <v>5</v>
       </c>
       <c r="J353">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K353">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L353">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M353">
         <v>3</v>
@@ -18506,19 +18506,19 @@
         <v>4</v>
       </c>
       <c r="J354">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K354">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L354">
         <v>4</v>
       </c>
       <c r="M354">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N354">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O354">
         <v>6</v>
@@ -18565,7 +18565,7 @@
         <v>3</v>
       </c>
       <c r="N355">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O355">
         <v>6</v>
@@ -18600,7 +18600,7 @@
         <v>6</v>
       </c>
       <c r="J356">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K356">
         <v>5</v>
@@ -18609,7 +18609,7 @@
         <v>5</v>
       </c>
       <c r="M356">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N356">
         <v>5</v>
@@ -18650,13 +18650,13 @@
         <v>3</v>
       </c>
       <c r="K357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N357">
         <v>3</v>
@@ -18741,7 +18741,7 @@
         <v>3</v>
       </c>
       <c r="J359">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K359">
         <v>4</v>
@@ -18750,10 +18750,10 @@
         <v>3</v>
       </c>
       <c r="M359">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N359">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O359">
         <v>6</v>
@@ -18794,7 +18794,7 @@
         <v>1</v>
       </c>
       <c r="L360">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M360">
         <v>3</v>
@@ -18835,19 +18835,19 @@
         <v>5</v>
       </c>
       <c r="J361">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K361">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L361">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M361">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N361">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O361">
         <v>6</v>
@@ -18882,19 +18882,19 @@
         <v>5</v>
       </c>
       <c r="J362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L362">
         <v>2</v>
       </c>
       <c r="M362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O362">
         <v>6</v>
@@ -18929,19 +18929,19 @@
         <v>6</v>
       </c>
       <c r="J363">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K363">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L363">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M363">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N363">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O363">
         <v>6</v>
@@ -18976,19 +18976,19 @@
         <v>6</v>
       </c>
       <c r="J364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M364">
         <v>3</v>
       </c>
       <c r="N364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O364">
         <v>6</v>
@@ -19023,19 +19023,19 @@
         <v>4</v>
       </c>
       <c r="J365">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K365">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L365">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M365">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N365">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O365">
         <v>6</v>
@@ -19120,16 +19120,16 @@
         <v>1</v>
       </c>
       <c r="K367">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L367">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M367">
         <v>2</v>
       </c>
       <c r="N367">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O367">
         <v>6</v>
@@ -19258,16 +19258,16 @@
         <v>4</v>
       </c>
       <c r="J370">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K370">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L370">
         <v>3</v>
       </c>
       <c r="M370">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N370">
         <v>3</v>
@@ -19352,7 +19352,7 @@
         <v>4</v>
       </c>
       <c r="J372">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K372">
         <v>4</v>
@@ -19361,7 +19361,7 @@
         <v>4</v>
       </c>
       <c r="M372">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N372">
         <v>4</v>
@@ -19399,19 +19399,19 @@
         <v>4</v>
       </c>
       <c r="J373">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K373">
         <v>4</v>
       </c>
       <c r="L373">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M373">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N373">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O373">
         <v>6</v>
@@ -19452,10 +19452,10 @@
         <v>3</v>
       </c>
       <c r="L374">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M374">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N374">
         <v>1</v>
@@ -19493,19 +19493,19 @@
         <v>4</v>
       </c>
       <c r="J375">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K375">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L375">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M375">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N375">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O375">
         <v>6</v>
@@ -19593,7 +19593,7 @@
         <v>2</v>
       </c>
       <c r="L377">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M377">
         <v>2</v>
@@ -19681,19 +19681,19 @@
         <v>3</v>
       </c>
       <c r="J379">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K379">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L379">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M379">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N379">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O379">
         <v>6</v>
@@ -19822,19 +19822,19 @@
         <v>6</v>
       </c>
       <c r="J382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K382">
         <v>5</v>
       </c>
       <c r="L382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O382">
         <v>6</v>
@@ -19963,16 +19963,16 @@
         <v>4</v>
       </c>
       <c r="J385">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K385">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L385">
         <v>4</v>
       </c>
       <c r="M385">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N385">
         <v>3</v>
@@ -20022,7 +20022,7 @@
         <v>3</v>
       </c>
       <c r="N386">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O386">
         <v>6</v>
@@ -20104,19 +20104,19 @@
         <v>6</v>
       </c>
       <c r="J388">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K388">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L388">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M388">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N388">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O388">
         <v>6</v>
@@ -20163,7 +20163,7 @@
         <v>3</v>
       </c>
       <c r="N389">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O389">
         <v>6</v>
@@ -20201,10 +20201,10 @@
         <v>3</v>
       </c>
       <c r="K390">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L390">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M390">
         <v>2</v>
@@ -20245,19 +20245,19 @@
         <v>7</v>
       </c>
       <c r="J391">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K391">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L391">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M391">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N391">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O391">
         <v>6</v>
@@ -20292,19 +20292,19 @@
         <v>4</v>
       </c>
       <c r="J392">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K392">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L392">
         <v>3</v>
       </c>
       <c r="M392">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N392">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O392">
         <v>6</v>
@@ -20339,13 +20339,13 @@
         <v>5</v>
       </c>
       <c r="J393">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K393">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L393">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M393">
         <v>2</v>
@@ -20433,13 +20433,13 @@
         <v>5</v>
       </c>
       <c r="J395">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K395">
         <v>2</v>
       </c>
       <c r="L395">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M395">
         <v>4</v>
@@ -20483,13 +20483,13 @@
         <v>5</v>
       </c>
       <c r="K396">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L396">
         <v>5</v>
       </c>
       <c r="M396">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N396">
         <v>5</v>
@@ -20577,13 +20577,13 @@
         <v>3</v>
       </c>
       <c r="K398">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L398">
         <v>2</v>
       </c>
       <c r="M398">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N398">
         <v>1</v>
@@ -20630,7 +20630,7 @@
         <v>1</v>
       </c>
       <c r="M399">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N399">
         <v>1</v>
@@ -20671,16 +20671,16 @@
         <v>3</v>
       </c>
       <c r="K400">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L400">
         <v>3</v>
       </c>
       <c r="M400">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N400">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O400">
         <v>6</v>
@@ -20762,7 +20762,7 @@
         <v>4</v>
       </c>
       <c r="J402">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K402">
         <v>5</v>

</xml_diff>

<commit_message>
fix(corr): BE-ME -0.08 ns (was -0.43***); sync data+results+raw_output
</commit_message>
<xml_diff>
--- a/data/T2_cleaned.xlsx
+++ b/data/T2_cleaned.xlsx
@@ -1962,19 +1962,19 @@
         <v>3</v>
       </c>
       <c r="J2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -2062,7 +2062,7 @@
         <v>3</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4">
         <v>2</v>
@@ -2109,7 +2109,7 @@
         <v>2</v>
       </c>
       <c r="L5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -2200,13 +2200,13 @@
         <v>2</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -2250,10 +2250,10 @@
         <v>3</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N8">
         <v>3</v>
@@ -2347,10 +2347,10 @@
         <v>4</v>
       </c>
       <c r="M10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -2526,16 +2526,16 @@
         <v>6</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K14">
         <v>3</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N14">
         <v>3</v>
@@ -2573,19 +2573,19 @@
         <v>5</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O15">
         <v>6</v>
@@ -2620,19 +2620,19 @@
         <v>5</v>
       </c>
       <c r="J16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16">
         <v>1</v>
       </c>
       <c r="N16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O16">
         <v>6</v>
@@ -2667,19 +2667,19 @@
         <v>5</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17">
         <v>2</v>
       </c>
       <c r="M17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -2761,16 +2761,16 @@
         <v>5</v>
       </c>
       <c r="J19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N19">
         <v>2</v>
@@ -2808,19 +2808,19 @@
         <v>4</v>
       </c>
       <c r="J20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2858,7 +2858,7 @@
         <v>4</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L21">
         <v>4</v>
@@ -2902,7 +2902,7 @@
         <v>5</v>
       </c>
       <c r="J22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K22">
         <v>4</v>
@@ -2911,7 +2911,7 @@
         <v>5</v>
       </c>
       <c r="M22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N22">
         <v>4</v>
@@ -2949,19 +2949,19 @@
         <v>3</v>
       </c>
       <c r="J23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L23">
         <v>4</v>
       </c>
       <c r="M23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O23">
         <v>6</v>
@@ -3093,7 +3093,7 @@
         <v>4</v>
       </c>
       <c r="K26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L26">
         <v>3</v>
@@ -3187,13 +3187,13 @@
         <v>3</v>
       </c>
       <c r="K28">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L28">
         <v>3</v>
       </c>
       <c r="M28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N28">
         <v>2</v>
@@ -3231,16 +3231,16 @@
         <v>4</v>
       </c>
       <c r="J29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N29">
         <v>5</v>
@@ -3325,16 +3325,16 @@
         <v>3</v>
       </c>
       <c r="J31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L31">
         <v>4</v>
       </c>
       <c r="M31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N31">
         <v>4</v>
@@ -3431,7 +3431,7 @@
         <v>2</v>
       </c>
       <c r="N33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -3469,10 +3469,10 @@
         <v>4</v>
       </c>
       <c r="K34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M34">
         <v>4</v>
@@ -3513,7 +3513,7 @@
         <v>5</v>
       </c>
       <c r="J35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K35">
         <v>3</v>
@@ -3522,10 +3522,10 @@
         <v>2</v>
       </c>
       <c r="M35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O35">
         <v>6</v>
@@ -3563,16 +3563,16 @@
         <v>4</v>
       </c>
       <c r="K36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -3607,19 +3607,19 @@
         <v>3</v>
       </c>
       <c r="J37">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N37">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -3657,7 +3657,7 @@
         <v>2</v>
       </c>
       <c r="K38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L38">
         <v>1</v>
@@ -3701,19 +3701,19 @@
         <v>2</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3845,13 +3845,13 @@
         <v>3</v>
       </c>
       <c r="K42">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N42">
         <v>2</v>
@@ -3989,7 +3989,7 @@
         <v>5</v>
       </c>
       <c r="L45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M45">
         <v>4</v>
@@ -4030,16 +4030,16 @@
         <v>4</v>
       </c>
       <c r="J46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N46">
         <v>4</v>
@@ -4077,19 +4077,19 @@
         <v>6</v>
       </c>
       <c r="J47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L47">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O47">
         <v>6</v>
@@ -4124,19 +4124,19 @@
         <v>7</v>
       </c>
       <c r="J48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K48">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M48">
         <v>3</v>
       </c>
       <c r="N48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O48">
         <v>6</v>
@@ -4174,7 +4174,7 @@
         <v>1</v>
       </c>
       <c r="K49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49">
         <v>1</v>
@@ -4218,19 +4218,19 @@
         <v>6</v>
       </c>
       <c r="J50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K50">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4315,13 +4315,13 @@
         <v>1</v>
       </c>
       <c r="K52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N52">
         <v>1</v>
@@ -4359,16 +4359,16 @@
         <v>7</v>
       </c>
       <c r="J53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L53">
         <v>4</v>
       </c>
       <c r="M53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N53">
         <v>2</v>
@@ -4409,16 +4409,16 @@
         <v>2</v>
       </c>
       <c r="K54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4506,7 +4506,7 @@
         <v>1</v>
       </c>
       <c r="L56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M56">
         <v>1</v>
@@ -4556,10 +4556,10 @@
         <v>3</v>
       </c>
       <c r="M57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4691,7 +4691,7 @@
         <v>3</v>
       </c>
       <c r="K60">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L60">
         <v>3</v>
@@ -4876,7 +4876,7 @@
         <v>3</v>
       </c>
       <c r="J64">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K64">
         <v>5</v>
@@ -4923,19 +4923,19 @@
         <v>3</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L65">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M65">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N65">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -4970,19 +4970,19 @@
         <v>7</v>
       </c>
       <c r="J66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5020,7 +5020,7 @@
         <v>4</v>
       </c>
       <c r="K67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L67">
         <v>3</v>
@@ -5158,19 +5158,19 @@
         <v>2</v>
       </c>
       <c r="J70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O70">
         <v>6</v>
@@ -5205,16 +5205,16 @@
         <v>3</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L71">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N71">
         <v>3</v>
@@ -5252,19 +5252,19 @@
         <v>4</v>
       </c>
       <c r="J72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K72">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N72">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O72">
         <v>6</v>
@@ -5299,19 +5299,19 @@
         <v>7</v>
       </c>
       <c r="J73">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5346,19 +5346,19 @@
         <v>7</v>
       </c>
       <c r="J74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5396,7 +5396,7 @@
         <v>1</v>
       </c>
       <c r="K75">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L75">
         <v>4</v>
@@ -5443,10 +5443,10 @@
         <v>2</v>
       </c>
       <c r="K76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M76">
         <v>1</v>
@@ -5487,19 +5487,19 @@
         <v>3</v>
       </c>
       <c r="J77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5546,7 +5546,7 @@
         <v>1</v>
       </c>
       <c r="N78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5581,7 +5581,7 @@
         <v>5</v>
       </c>
       <c r="J79">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K79">
         <v>4</v>
@@ -5593,7 +5593,7 @@
         <v>4</v>
       </c>
       <c r="N79">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -5628,19 +5628,19 @@
         <v>7</v>
       </c>
       <c r="J80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O80">
         <v>6</v>
@@ -5772,7 +5772,7 @@
         <v>3</v>
       </c>
       <c r="K83">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L83">
         <v>3</v>
@@ -5816,19 +5816,19 @@
         <v>4</v>
       </c>
       <c r="J84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K84">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O84">
         <v>6</v>
@@ -5863,19 +5863,19 @@
         <v>2</v>
       </c>
       <c r="J85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K85">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N85">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O85">
         <v>6</v>
@@ -5910,19 +5910,19 @@
         <v>7</v>
       </c>
       <c r="J86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L86">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M86">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N86">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O86">
         <v>6</v>
@@ -6007,13 +6007,13 @@
         <v>2</v>
       </c>
       <c r="K88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L88">
         <v>3</v>
       </c>
       <c r="M88">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N88">
         <v>2</v>
@@ -6051,19 +6051,19 @@
         <v>4</v>
       </c>
       <c r="J89">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M89">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N89">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O89">
         <v>6</v>
@@ -6098,19 +6098,19 @@
         <v>7</v>
       </c>
       <c r="J90">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L90">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M90">
         <v>3</v>
       </c>
       <c r="N90">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O90">
         <v>6</v>
@@ -6145,19 +6145,19 @@
         <v>7</v>
       </c>
       <c r="J91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K91">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L91">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M91">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O91">
         <v>6</v>
@@ -6239,19 +6239,19 @@
         <v>4</v>
       </c>
       <c r="J93">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K93">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L93">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M93">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N93">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O93">
         <v>6</v>
@@ -6286,19 +6286,19 @@
         <v>5</v>
       </c>
       <c r="J94">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K94">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L94">
         <v>2</v>
       </c>
       <c r="M94">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N94">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O94">
         <v>6</v>
@@ -6383,16 +6383,16 @@
         <v>1</v>
       </c>
       <c r="K96">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M96">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N96">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O96">
         <v>6</v>
@@ -6521,16 +6521,16 @@
         <v>3</v>
       </c>
       <c r="J99">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K99">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L99">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M99">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N99">
         <v>3</v>
@@ -6574,7 +6574,7 @@
         <v>3</v>
       </c>
       <c r="L100">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M100">
         <v>6</v>
@@ -6615,19 +6615,19 @@
         <v>6</v>
       </c>
       <c r="J101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K101">
         <v>3</v>
       </c>
       <c r="L101">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N101">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O101">
         <v>6</v>
@@ -6712,16 +6712,16 @@
         <v>4</v>
       </c>
       <c r="K103">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L103">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M103">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N103">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O103">
         <v>6</v>
@@ -6756,19 +6756,19 @@
         <v>6</v>
       </c>
       <c r="J104">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K104">
         <v>1</v>
       </c>
       <c r="L104">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M104">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N104">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O104">
         <v>6</v>
@@ -6803,16 +6803,16 @@
         <v>7</v>
       </c>
       <c r="J105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K105">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L105">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M105">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N105">
         <v>1</v>
@@ -6897,7 +6897,7 @@
         <v>5</v>
       </c>
       <c r="J107">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K107">
         <v>3</v>
@@ -7000,7 +7000,7 @@
         <v>1</v>
       </c>
       <c r="M109">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N109">
         <v>2</v>
@@ -7038,19 +7038,19 @@
         <v>1</v>
       </c>
       <c r="J110">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K110">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L110">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M110">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N110">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O110">
         <v>6</v>
@@ -7132,19 +7132,19 @@
         <v>4</v>
       </c>
       <c r="J112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M112">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N112">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O112">
         <v>6</v>
@@ -7179,13 +7179,13 @@
         <v>4</v>
       </c>
       <c r="J113">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K113">
         <v>1</v>
       </c>
       <c r="L113">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M113">
         <v>1</v>
@@ -7273,19 +7273,19 @@
         <v>3</v>
       </c>
       <c r="J115">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K115">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L115">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M115">
         <v>4</v>
       </c>
       <c r="N115">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O115">
         <v>6</v>
@@ -7320,19 +7320,19 @@
         <v>3</v>
       </c>
       <c r="J116">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K116">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L116">
         <v>3</v>
       </c>
       <c r="M116">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N116">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O116">
         <v>6</v>
@@ -7367,7 +7367,7 @@
         <v>4</v>
       </c>
       <c r="J117">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K117">
         <v>3</v>
@@ -7379,7 +7379,7 @@
         <v>4</v>
       </c>
       <c r="N117">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O117">
         <v>6</v>
@@ -7558,13 +7558,13 @@
         <v>3</v>
       </c>
       <c r="K121">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L121">
         <v>3</v>
       </c>
       <c r="M121">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N121">
         <v>4</v>
@@ -7602,13 +7602,13 @@
         <v>6</v>
       </c>
       <c r="J122">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K122">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L122">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M122">
         <v>5</v>
@@ -7802,7 +7802,7 @@
         <v>2</v>
       </c>
       <c r="N126">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O126">
         <v>6</v>
@@ -7849,7 +7849,7 @@
         <v>5</v>
       </c>
       <c r="N127">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O127">
         <v>6</v>
@@ -7931,13 +7931,13 @@
         <v>4</v>
       </c>
       <c r="J129">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K129">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L129">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M129">
         <v>7</v>
@@ -7978,19 +7978,19 @@
         <v>7</v>
       </c>
       <c r="J130">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K130">
         <v>3</v>
       </c>
       <c r="L130">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M130">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N130">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O130">
         <v>6</v>
@@ -8072,19 +8072,19 @@
         <v>5</v>
       </c>
       <c r="J132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M132">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N132">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O132">
         <v>6</v>
@@ -8119,19 +8119,19 @@
         <v>3</v>
       </c>
       <c r="J133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M133">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N133">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O133">
         <v>6</v>
@@ -8166,19 +8166,19 @@
         <v>2</v>
       </c>
       <c r="J134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N134">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O134">
         <v>6</v>
@@ -8260,19 +8260,19 @@
         <v>6</v>
       </c>
       <c r="J136">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K136">
         <v>3</v>
       </c>
       <c r="L136">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M136">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N136">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O136">
         <v>6</v>
@@ -8307,19 +8307,19 @@
         <v>3</v>
       </c>
       <c r="J137">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K137">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L137">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M137">
         <v>2</v>
       </c>
       <c r="N137">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O137">
         <v>6</v>
@@ -8354,19 +8354,19 @@
         <v>4</v>
       </c>
       <c r="J138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K138">
         <v>3</v>
       </c>
       <c r="L138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M138">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N138">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O138">
         <v>6</v>
@@ -8404,7 +8404,7 @@
         <v>4</v>
       </c>
       <c r="K139">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L139">
         <v>3</v>
@@ -8448,19 +8448,19 @@
         <v>5</v>
       </c>
       <c r="J140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K140">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L140">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N140">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O140">
         <v>6</v>
@@ -8592,7 +8592,7 @@
         <v>4</v>
       </c>
       <c r="K143">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L143">
         <v>3</v>
@@ -8636,7 +8636,7 @@
         <v>5</v>
       </c>
       <c r="J144">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K144">
         <v>5</v>
@@ -8739,7 +8739,7 @@
         <v>3</v>
       </c>
       <c r="M146">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N146">
         <v>4</v>
@@ -8777,19 +8777,19 @@
         <v>6</v>
       </c>
       <c r="J147">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K147">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L147">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M147">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N147">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O147">
         <v>6</v>
@@ -8830,7 +8830,7 @@
         <v>3</v>
       </c>
       <c r="L148">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M148">
         <v>4</v>
@@ -8883,7 +8883,7 @@
         <v>4</v>
       </c>
       <c r="N149">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O149">
         <v>6</v>
@@ -8921,16 +8921,16 @@
         <v>6</v>
       </c>
       <c r="K150">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L150">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M150">
         <v>4</v>
       </c>
       <c r="N150">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O150">
         <v>6</v>
@@ -8968,16 +8968,16 @@
         <v>1</v>
       </c>
       <c r="K151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N151">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O151">
         <v>6</v>
@@ -9109,10 +9109,10 @@
         <v>1</v>
       </c>
       <c r="K154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L154">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M154">
         <v>1</v>
@@ -9162,7 +9162,7 @@
         <v>4</v>
       </c>
       <c r="M155">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N155">
         <v>2</v>
@@ -9200,7 +9200,7 @@
         <v>6</v>
       </c>
       <c r="J156">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K156">
         <v>3</v>
@@ -9209,7 +9209,7 @@
         <v>3</v>
       </c>
       <c r="M156">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N156">
         <v>4</v>
@@ -9247,19 +9247,19 @@
         <v>7</v>
       </c>
       <c r="J157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K157">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M157">
         <v>3</v>
       </c>
       <c r="N157">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O157">
         <v>6</v>
@@ -9297,16 +9297,16 @@
         <v>4</v>
       </c>
       <c r="K158">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L158">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M158">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N158">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O158">
         <v>6</v>
@@ -9400,7 +9400,7 @@
         <v>3</v>
       </c>
       <c r="N160">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O160">
         <v>6</v>
@@ -9435,19 +9435,19 @@
         <v>3</v>
       </c>
       <c r="J161">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K161">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L161">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M161">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N161">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O161">
         <v>6</v>
@@ -9541,7 +9541,7 @@
         <v>1</v>
       </c>
       <c r="N163">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O163">
         <v>6</v>
@@ -9579,7 +9579,7 @@
         <v>3</v>
       </c>
       <c r="K164">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L164">
         <v>3</v>
@@ -9673,13 +9673,13 @@
         <v>3</v>
       </c>
       <c r="K166">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L166">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M166">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N166">
         <v>3</v>
@@ -9764,10 +9764,10 @@
         <v>5</v>
       </c>
       <c r="J168">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K168">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L168">
         <v>3</v>
@@ -9858,19 +9858,19 @@
         <v>4</v>
       </c>
       <c r="J170">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K170">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L170">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M170">
         <v>4</v>
       </c>
       <c r="N170">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O170">
         <v>6</v>
@@ -9905,19 +9905,19 @@
         <v>5</v>
       </c>
       <c r="J171">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K171">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L171">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M171">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N171">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O171">
         <v>6</v>
@@ -9952,19 +9952,19 @@
         <v>6</v>
       </c>
       <c r="J172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K172">
         <v>3</v>
       </c>
       <c r="L172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M172">
         <v>4</v>
       </c>
       <c r="N172">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O172">
         <v>6</v>
@@ -9999,19 +9999,19 @@
         <v>5</v>
       </c>
       <c r="J173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K173">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M173">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N173">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O173">
         <v>6</v>
@@ -10055,7 +10055,7 @@
         <v>3</v>
       </c>
       <c r="M174">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N174">
         <v>2</v>
@@ -10140,7 +10140,7 @@
         <v>6</v>
       </c>
       <c r="J176">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K176">
         <v>1</v>
@@ -10293,7 +10293,7 @@
         <v>3</v>
       </c>
       <c r="N179">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O179">
         <v>6</v>
@@ -10331,7 +10331,7 @@
         <v>3</v>
       </c>
       <c r="K180">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L180">
         <v>4</v>
@@ -10469,10 +10469,10 @@
         <v>5</v>
       </c>
       <c r="J183">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K183">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L183">
         <v>1</v>
@@ -10516,19 +10516,19 @@
         <v>5</v>
       </c>
       <c r="J184">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K184">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L184">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M184">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N184">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O184">
         <v>6</v>
@@ -10569,10 +10569,10 @@
         <v>4</v>
       </c>
       <c r="L185">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M185">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N185">
         <v>3</v>
@@ -10619,10 +10619,10 @@
         <v>5</v>
       </c>
       <c r="M186">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N186">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O186">
         <v>6</v>
@@ -10657,16 +10657,16 @@
         <v>4</v>
       </c>
       <c r="J187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K187">
         <v>3</v>
       </c>
       <c r="L187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M187">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N187">
         <v>4</v>
@@ -10986,19 +10986,19 @@
         <v>7</v>
       </c>
       <c r="J194">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K194">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L194">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M194">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N194">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O194">
         <v>6</v>
@@ -11036,10 +11036,10 @@
         <v>4</v>
       </c>
       <c r="K195">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L195">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M195">
         <v>5</v>
@@ -11080,19 +11080,19 @@
         <v>1</v>
       </c>
       <c r="J196">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K196">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L196">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M196">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N196">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O196">
         <v>6</v>
@@ -11127,10 +11127,10 @@
         <v>4</v>
       </c>
       <c r="J197">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K197">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L197">
         <v>4</v>
@@ -11174,7 +11174,7 @@
         <v>3</v>
       </c>
       <c r="J198">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K198">
         <v>5</v>
@@ -11268,16 +11268,16 @@
         <v>6</v>
       </c>
       <c r="J200">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K200">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L200">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M200">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N200">
         <v>4</v>
@@ -11315,19 +11315,19 @@
         <v>3</v>
       </c>
       <c r="J201">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K201">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L201">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M201">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N201">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O201">
         <v>6</v>
@@ -11362,19 +11362,19 @@
         <v>2</v>
       </c>
       <c r="J202">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K202">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L202">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M202">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N202">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O202">
         <v>6</v>
@@ -11409,7 +11409,7 @@
         <v>2</v>
       </c>
       <c r="J203">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K203">
         <v>2</v>
@@ -11456,19 +11456,19 @@
         <v>4</v>
       </c>
       <c r="J204">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K204">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L204">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M204">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N204">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O204">
         <v>6</v>
@@ -11512,10 +11512,10 @@
         <v>5</v>
       </c>
       <c r="M205">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N205">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O205">
         <v>6</v>
@@ -11550,19 +11550,19 @@
         <v>4</v>
       </c>
       <c r="J206">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K206">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L206">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M206">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N206">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O206">
         <v>6</v>
@@ -11600,7 +11600,7 @@
         <v>4</v>
       </c>
       <c r="K207">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L207">
         <v>4</v>
@@ -11644,10 +11644,10 @@
         <v>4</v>
       </c>
       <c r="J208">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K208">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L208">
         <v>2</v>
@@ -11656,7 +11656,7 @@
         <v>2</v>
       </c>
       <c r="N208">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O208">
         <v>6</v>
@@ -11700,7 +11700,7 @@
         <v>3</v>
       </c>
       <c r="M209">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N209">
         <v>3</v>
@@ -11785,19 +11785,19 @@
         <v>1</v>
       </c>
       <c r="J211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N211">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O211">
         <v>6</v>
@@ -11835,16 +11835,16 @@
         <v>4</v>
       </c>
       <c r="K212">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L212">
         <v>4</v>
       </c>
       <c r="M212">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N212">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O212">
         <v>6</v>
@@ -11926,7 +11926,7 @@
         <v>5</v>
       </c>
       <c r="J214">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K214">
         <v>2</v>
@@ -11976,7 +11976,7 @@
         <v>2</v>
       </c>
       <c r="K215">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L215">
         <v>1</v>
@@ -11985,7 +11985,7 @@
         <v>4</v>
       </c>
       <c r="N215">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O215">
         <v>6</v>
@@ -12076,10 +12076,10 @@
         <v>3</v>
       </c>
       <c r="M217">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N217">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O217">
         <v>6</v>
@@ -12161,16 +12161,16 @@
         <v>3</v>
       </c>
       <c r="J219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M219">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N219">
         <v>1</v>
@@ -12264,7 +12264,7 @@
         <v>2</v>
       </c>
       <c r="M221">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N221">
         <v>1</v>
@@ -12349,19 +12349,19 @@
         <v>4</v>
       </c>
       <c r="J223">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K223">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L223">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M223">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N223">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O223">
         <v>6</v>
@@ -12443,10 +12443,10 @@
         <v>3</v>
       </c>
       <c r="J225">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K225">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L225">
         <v>2</v>
@@ -12455,7 +12455,7 @@
         <v>2</v>
       </c>
       <c r="N225">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O225">
         <v>6</v>
@@ -12502,7 +12502,7 @@
         <v>1</v>
       </c>
       <c r="N226">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O226">
         <v>6</v>
@@ -12584,10 +12584,10 @@
         <v>6</v>
       </c>
       <c r="J228">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K228">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L228">
         <v>2</v>
@@ -12596,7 +12596,7 @@
         <v>2</v>
       </c>
       <c r="N228">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O228">
         <v>6</v>
@@ -12637,7 +12637,7 @@
         <v>2</v>
       </c>
       <c r="L229">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M229">
         <v>1</v>
@@ -12731,7 +12731,7 @@
         <v>2</v>
       </c>
       <c r="L231">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M231">
         <v>1</v>
@@ -12866,19 +12866,19 @@
         <v>5</v>
       </c>
       <c r="J234">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K234">
         <v>3</v>
       </c>
       <c r="L234">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M234">
         <v>3</v>
       </c>
       <c r="N234">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O234">
         <v>6</v>
@@ -12913,16 +12913,16 @@
         <v>5</v>
       </c>
       <c r="J235">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K235">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L235">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M235">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N235">
         <v>3</v>
@@ -12960,19 +12960,19 @@
         <v>5</v>
       </c>
       <c r="J236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M236">
         <v>3</v>
       </c>
       <c r="N236">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O236">
         <v>6</v>
@@ -13007,19 +13007,19 @@
         <v>6</v>
       </c>
       <c r="J237">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K237">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L237">
         <v>4</v>
       </c>
       <c r="M237">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N237">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O237">
         <v>6</v>
@@ -13054,10 +13054,10 @@
         <v>6</v>
       </c>
       <c r="J238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L238">
         <v>3</v>
@@ -13066,7 +13066,7 @@
         <v>1</v>
       </c>
       <c r="N238">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O238">
         <v>6</v>
@@ -13107,7 +13107,7 @@
         <v>2</v>
       </c>
       <c r="L239">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M239">
         <v>2</v>
@@ -13160,7 +13160,7 @@
         <v>5</v>
       </c>
       <c r="N240">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O240">
         <v>6</v>
@@ -13195,19 +13195,19 @@
         <v>4</v>
       </c>
       <c r="J241">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K241">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L241">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M241">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N241">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O241">
         <v>6</v>
@@ -13242,19 +13242,19 @@
         <v>5</v>
       </c>
       <c r="J242">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M242">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N242">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O242">
         <v>6</v>
@@ -13295,7 +13295,7 @@
         <v>3</v>
       </c>
       <c r="L243">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M243">
         <v>2</v>
@@ -13436,7 +13436,7 @@
         <v>1</v>
       </c>
       <c r="L246">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M246">
         <v>1</v>
@@ -13536,7 +13536,7 @@
         <v>1</v>
       </c>
       <c r="N248">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O248">
         <v>6</v>
@@ -13580,7 +13580,7 @@
         <v>1</v>
       </c>
       <c r="M249">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N249">
         <v>2</v>
@@ -13624,10 +13624,10 @@
         <v>5</v>
       </c>
       <c r="L250">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M250">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N250">
         <v>5</v>
@@ -13859,7 +13859,7 @@
         <v>4</v>
       </c>
       <c r="L255">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M255">
         <v>4</v>
@@ -13994,19 +13994,19 @@
         <v>4</v>
       </c>
       <c r="J258">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K258">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L258">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M258">
         <v>2</v>
       </c>
       <c r="N258">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O258">
         <v>6</v>
@@ -14088,19 +14088,19 @@
         <v>4</v>
       </c>
       <c r="J260">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K260">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L260">
         <v>5</v>
       </c>
       <c r="M260">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N260">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O260">
         <v>6</v>
@@ -14182,13 +14182,13 @@
         <v>1</v>
       </c>
       <c r="J262">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K262">
         <v>3</v>
       </c>
       <c r="L262">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M262">
         <v>4</v>
@@ -14232,16 +14232,16 @@
         <v>4</v>
       </c>
       <c r="K263">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L263">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M263">
         <v>4</v>
       </c>
       <c r="N263">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O263">
         <v>6</v>
@@ -14376,10 +14376,10 @@
         <v>1</v>
       </c>
       <c r="L266">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M266">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N266">
         <v>1</v>
@@ -14417,16 +14417,16 @@
         <v>4</v>
       </c>
       <c r="J267">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K267">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L267">
         <v>2</v>
       </c>
       <c r="M267">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N267">
         <v>3</v>
@@ -14470,7 +14470,7 @@
         <v>5</v>
       </c>
       <c r="L268">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M268">
         <v>6</v>
@@ -14511,19 +14511,19 @@
         <v>7</v>
       </c>
       <c r="J269">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K269">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L269">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M269">
         <v>3</v>
       </c>
       <c r="N269">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O269">
         <v>6</v>
@@ -14558,7 +14558,7 @@
         <v>7</v>
       </c>
       <c r="J270">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K270">
         <v>3</v>
@@ -14614,7 +14614,7 @@
         <v>1</v>
       </c>
       <c r="M271">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N271">
         <v>1</v>
@@ -14708,7 +14708,7 @@
         <v>2</v>
       </c>
       <c r="M273">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N273">
         <v>4</v>
@@ -14746,13 +14746,13 @@
         <v>3</v>
       </c>
       <c r="J274">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K274">
         <v>2</v>
       </c>
       <c r="L274">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M274">
         <v>2</v>
@@ -14840,16 +14840,16 @@
         <v>3</v>
       </c>
       <c r="J276">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K276">
         <v>4</v>
       </c>
       <c r="L276">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M276">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N276">
         <v>6</v>
@@ -14896,10 +14896,10 @@
         <v>4</v>
       </c>
       <c r="M277">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N277">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O277">
         <v>6</v>
@@ -14981,19 +14981,19 @@
         <v>6</v>
       </c>
       <c r="J279">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K279">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L279">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M279">
         <v>4</v>
       </c>
       <c r="N279">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O279">
         <v>6</v>
@@ -15028,7 +15028,7 @@
         <v>3</v>
       </c>
       <c r="J280">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K280">
         <v>1</v>
@@ -15037,10 +15037,10 @@
         <v>2</v>
       </c>
       <c r="M280">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N280">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O280">
         <v>6</v>
@@ -15078,7 +15078,7 @@
         <v>4</v>
       </c>
       <c r="K281">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L281">
         <v>3</v>
@@ -15134,7 +15134,7 @@
         <v>3</v>
       </c>
       <c r="N282">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O282">
         <v>6</v>
@@ -15169,7 +15169,7 @@
         <v>4</v>
       </c>
       <c r="J283">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K283">
         <v>2</v>
@@ -15216,19 +15216,19 @@
         <v>7</v>
       </c>
       <c r="J284">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K284">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L284">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M284">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N284">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O284">
         <v>6</v>
@@ -15313,7 +15313,7 @@
         <v>6</v>
       </c>
       <c r="K286">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L286">
         <v>6</v>
@@ -15366,7 +15366,7 @@
         <v>1</v>
       </c>
       <c r="M287">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N287">
         <v>1</v>
@@ -15451,7 +15451,7 @@
         <v>3</v>
       </c>
       <c r="J289">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K289">
         <v>1</v>
@@ -15504,13 +15504,13 @@
         <v>4</v>
       </c>
       <c r="L290">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M290">
         <v>6</v>
       </c>
       <c r="N290">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O290">
         <v>6</v>
@@ -15545,19 +15545,19 @@
         <v>2</v>
       </c>
       <c r="J291">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K291">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L291">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M291">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N291">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O291">
         <v>6</v>
@@ -15595,13 +15595,13 @@
         <v>3</v>
       </c>
       <c r="K292">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L292">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M292">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N292">
         <v>2</v>
@@ -15639,19 +15639,19 @@
         <v>5</v>
       </c>
       <c r="J293">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K293">
         <v>4</v>
       </c>
       <c r="L293">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M293">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N293">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O293">
         <v>6</v>
@@ -15780,19 +15780,19 @@
         <v>3</v>
       </c>
       <c r="J296">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K296">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L296">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M296">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N296">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O296">
         <v>6</v>
@@ -15830,7 +15830,7 @@
         <v>2</v>
       </c>
       <c r="K297">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L297">
         <v>2</v>
@@ -15839,7 +15839,7 @@
         <v>3</v>
       </c>
       <c r="N297">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O297">
         <v>6</v>
@@ -15874,19 +15874,19 @@
         <v>3</v>
       </c>
       <c r="J298">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K298">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L298">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M298">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N298">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O298">
         <v>6</v>
@@ -15924,16 +15924,16 @@
         <v>4</v>
       </c>
       <c r="K299">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L299">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M299">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N299">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O299">
         <v>6</v>
@@ -15968,19 +15968,19 @@
         <v>5</v>
       </c>
       <c r="J300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L300">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N300">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O300">
         <v>6</v>
@@ -16015,19 +16015,19 @@
         <v>7</v>
       </c>
       <c r="J301">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K301">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L301">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M301">
         <v>2</v>
       </c>
       <c r="N301">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O301">
         <v>6</v>
@@ -16112,16 +16112,16 @@
         <v>2</v>
       </c>
       <c r="K303">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L303">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M303">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N303">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O303">
         <v>6</v>
@@ -16156,19 +16156,19 @@
         <v>3</v>
       </c>
       <c r="J304">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K304">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L304">
         <v>4</v>
       </c>
       <c r="M304">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N304">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O304">
         <v>6</v>
@@ -16203,19 +16203,19 @@
         <v>6</v>
       </c>
       <c r="J305">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K305">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L305">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M305">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N305">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O305">
         <v>6</v>
@@ -16250,19 +16250,19 @@
         <v>6</v>
       </c>
       <c r="J306">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K306">
         <v>3</v>
       </c>
       <c r="L306">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M306">
         <v>4</v>
       </c>
       <c r="N306">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O306">
         <v>6</v>
@@ -16300,16 +16300,16 @@
         <v>2</v>
       </c>
       <c r="K307">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L307">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M307">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N307">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O307">
         <v>6</v>
@@ -16347,7 +16347,7 @@
         <v>3</v>
       </c>
       <c r="K308">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L308">
         <v>3</v>
@@ -16391,19 +16391,19 @@
         <v>4</v>
       </c>
       <c r="J309">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K309">
         <v>3</v>
       </c>
       <c r="L309">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M309">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N309">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O309">
         <v>6</v>
@@ -16485,7 +16485,7 @@
         <v>5</v>
       </c>
       <c r="J311">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K311">
         <v>4</v>
@@ -16582,13 +16582,13 @@
         <v>2</v>
       </c>
       <c r="K313">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L313">
         <v>3</v>
       </c>
       <c r="M313">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N313">
         <v>2</v>
@@ -16635,10 +16635,10 @@
         <v>4</v>
       </c>
       <c r="M314">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N314">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O314">
         <v>6</v>
@@ -16673,13 +16673,13 @@
         <v>6</v>
       </c>
       <c r="J315">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K315">
         <v>4</v>
       </c>
       <c r="L315">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M315">
         <v>3</v>
@@ -16720,19 +16720,19 @@
         <v>6</v>
       </c>
       <c r="J316">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M316">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N316">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O316">
         <v>6</v>
@@ -16814,19 +16814,19 @@
         <v>6</v>
       </c>
       <c r="J318">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K318">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L318">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M318">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N318">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O318">
         <v>6</v>
@@ -16864,13 +16864,13 @@
         <v>4</v>
       </c>
       <c r="K319">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L319">
         <v>4</v>
       </c>
       <c r="M319">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N319">
         <v>4</v>
@@ -16911,16 +16911,16 @@
         <v>1</v>
       </c>
       <c r="K320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M320">
         <v>1</v>
       </c>
       <c r="N320">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O320">
         <v>6</v>
@@ -17143,19 +17143,19 @@
         <v>3</v>
       </c>
       <c r="J325">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K325">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L325">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M325">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N325">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O325">
         <v>6</v>
@@ -17237,19 +17237,19 @@
         <v>4</v>
       </c>
       <c r="J327">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K327">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L327">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M327">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N327">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O327">
         <v>6</v>
@@ -17284,7 +17284,7 @@
         <v>6</v>
       </c>
       <c r="J328">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K328">
         <v>2</v>
@@ -17296,7 +17296,7 @@
         <v>5</v>
       </c>
       <c r="N328">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O328">
         <v>6</v>
@@ -17331,16 +17331,16 @@
         <v>4</v>
       </c>
       <c r="J329">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K329">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L329">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M329">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N329">
         <v>1</v>
@@ -17384,13 +17384,13 @@
         <v>2</v>
       </c>
       <c r="L330">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M330">
         <v>3</v>
       </c>
       <c r="N330">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O330">
         <v>6</v>
@@ -17425,19 +17425,19 @@
         <v>7</v>
       </c>
       <c r="J331">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K331">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L331">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M331">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N331">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O331">
         <v>6</v>
@@ -17472,16 +17472,16 @@
         <v>4</v>
       </c>
       <c r="J332">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K332">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L332">
         <v>4</v>
       </c>
       <c r="M332">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N332">
         <v>4</v>
@@ -17519,19 +17519,19 @@
         <v>6</v>
       </c>
       <c r="J333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L333">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N333">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O333">
         <v>6</v>
@@ -17566,7 +17566,7 @@
         <v>5</v>
       </c>
       <c r="J334">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K334">
         <v>2</v>
@@ -17660,19 +17660,19 @@
         <v>6</v>
       </c>
       <c r="J336">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K336">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L336">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M336">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N336">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O336">
         <v>6</v>
@@ -17707,19 +17707,19 @@
         <v>3</v>
       </c>
       <c r="J337">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K337">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L337">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M337">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N337">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O337">
         <v>6</v>
@@ -17804,7 +17804,7 @@
         <v>3</v>
       </c>
       <c r="K339">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L339">
         <v>4</v>
@@ -17895,19 +17895,19 @@
         <v>5</v>
       </c>
       <c r="J341">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K341">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L341">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M341">
         <v>2</v>
       </c>
       <c r="N341">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O341">
         <v>6</v>
@@ -18036,19 +18036,19 @@
         <v>3</v>
       </c>
       <c r="J344">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K344">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L344">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M344">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N344">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O344">
         <v>6</v>
@@ -18083,10 +18083,10 @@
         <v>5</v>
       </c>
       <c r="J345">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K345">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L345">
         <v>5</v>
@@ -18139,7 +18139,7 @@
         <v>4</v>
       </c>
       <c r="M346">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N346">
         <v>4</v>
@@ -18180,13 +18180,13 @@
         <v>2</v>
       </c>
       <c r="K347">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L347">
         <v>2</v>
       </c>
       <c r="M347">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N347">
         <v>1</v>
@@ -18283,7 +18283,7 @@
         <v>4</v>
       </c>
       <c r="N349">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O349">
         <v>6</v>
@@ -18327,7 +18327,7 @@
         <v>4</v>
       </c>
       <c r="M350">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N350">
         <v>4</v>
@@ -18412,19 +18412,19 @@
         <v>7</v>
       </c>
       <c r="J352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K352">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M352">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N352">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O352">
         <v>6</v>
@@ -18459,13 +18459,13 @@
         <v>5</v>
       </c>
       <c r="J353">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K353">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L353">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M353">
         <v>3</v>
@@ -18506,19 +18506,19 @@
         <v>4</v>
       </c>
       <c r="J354">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K354">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L354">
         <v>4</v>
       </c>
       <c r="M354">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N354">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O354">
         <v>6</v>
@@ -18565,7 +18565,7 @@
         <v>3</v>
       </c>
       <c r="N355">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O355">
         <v>6</v>
@@ -18600,7 +18600,7 @@
         <v>6</v>
       </c>
       <c r="J356">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K356">
         <v>5</v>
@@ -18609,7 +18609,7 @@
         <v>5</v>
       </c>
       <c r="M356">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N356">
         <v>5</v>
@@ -18650,13 +18650,13 @@
         <v>3</v>
       </c>
       <c r="K357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M357">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N357">
         <v>3</v>
@@ -18741,7 +18741,7 @@
         <v>3</v>
       </c>
       <c r="J359">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K359">
         <v>4</v>
@@ -18750,10 +18750,10 @@
         <v>3</v>
       </c>
       <c r="M359">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N359">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O359">
         <v>6</v>
@@ -18794,7 +18794,7 @@
         <v>1</v>
       </c>
       <c r="L360">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M360">
         <v>3</v>
@@ -18835,19 +18835,19 @@
         <v>5</v>
       </c>
       <c r="J361">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K361">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L361">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M361">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N361">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O361">
         <v>6</v>
@@ -18882,19 +18882,19 @@
         <v>5</v>
       </c>
       <c r="J362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L362">
         <v>2</v>
       </c>
       <c r="M362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N362">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O362">
         <v>6</v>
@@ -18929,19 +18929,19 @@
         <v>6</v>
       </c>
       <c r="J363">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K363">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L363">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M363">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N363">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O363">
         <v>6</v>
@@ -18976,19 +18976,19 @@
         <v>6</v>
       </c>
       <c r="J364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M364">
         <v>3</v>
       </c>
       <c r="N364">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O364">
         <v>6</v>
@@ -19023,19 +19023,19 @@
         <v>4</v>
       </c>
       <c r="J365">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K365">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L365">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M365">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N365">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O365">
         <v>6</v>
@@ -19120,16 +19120,16 @@
         <v>1</v>
       </c>
       <c r="K367">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L367">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M367">
         <v>2</v>
       </c>
       <c r="N367">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O367">
         <v>6</v>
@@ -19258,16 +19258,16 @@
         <v>4</v>
       </c>
       <c r="J370">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K370">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L370">
         <v>3</v>
       </c>
       <c r="M370">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N370">
         <v>3</v>
@@ -19352,7 +19352,7 @@
         <v>4</v>
       </c>
       <c r="J372">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K372">
         <v>4</v>
@@ -19361,7 +19361,7 @@
         <v>4</v>
       </c>
       <c r="M372">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N372">
         <v>4</v>
@@ -19399,19 +19399,19 @@
         <v>4</v>
       </c>
       <c r="J373">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K373">
         <v>4</v>
       </c>
       <c r="L373">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M373">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N373">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O373">
         <v>6</v>
@@ -19452,10 +19452,10 @@
         <v>3</v>
       </c>
       <c r="L374">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M374">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N374">
         <v>1</v>
@@ -19493,19 +19493,19 @@
         <v>4</v>
       </c>
       <c r="J375">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K375">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L375">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M375">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N375">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O375">
         <v>6</v>
@@ -19593,7 +19593,7 @@
         <v>2</v>
       </c>
       <c r="L377">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M377">
         <v>2</v>
@@ -19681,19 +19681,19 @@
         <v>3</v>
       </c>
       <c r="J379">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K379">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L379">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M379">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N379">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O379">
         <v>6</v>
@@ -19822,19 +19822,19 @@
         <v>6</v>
       </c>
       <c r="J382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K382">
         <v>5</v>
       </c>
       <c r="L382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N382">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O382">
         <v>6</v>
@@ -19963,16 +19963,16 @@
         <v>4</v>
       </c>
       <c r="J385">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K385">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L385">
         <v>4</v>
       </c>
       <c r="M385">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N385">
         <v>3</v>
@@ -20022,7 +20022,7 @@
         <v>3</v>
       </c>
       <c r="N386">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O386">
         <v>6</v>
@@ -20104,19 +20104,19 @@
         <v>6</v>
       </c>
       <c r="J388">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K388">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L388">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M388">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N388">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O388">
         <v>6</v>
@@ -20163,7 +20163,7 @@
         <v>3</v>
       </c>
       <c r="N389">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O389">
         <v>6</v>
@@ -20201,10 +20201,10 @@
         <v>3</v>
       </c>
       <c r="K390">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L390">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M390">
         <v>2</v>
@@ -20245,19 +20245,19 @@
         <v>7</v>
       </c>
       <c r="J391">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K391">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L391">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M391">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N391">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O391">
         <v>6</v>
@@ -20292,19 +20292,19 @@
         <v>4</v>
       </c>
       <c r="J392">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K392">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L392">
         <v>3</v>
       </c>
       <c r="M392">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N392">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O392">
         <v>6</v>
@@ -20339,13 +20339,13 @@
         <v>5</v>
       </c>
       <c r="J393">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K393">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L393">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M393">
         <v>2</v>
@@ -20433,13 +20433,13 @@
         <v>5</v>
       </c>
       <c r="J395">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K395">
         <v>2</v>
       </c>
       <c r="L395">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M395">
         <v>4</v>
@@ -20483,13 +20483,13 @@
         <v>5</v>
       </c>
       <c r="K396">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L396">
         <v>5</v>
       </c>
       <c r="M396">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N396">
         <v>5</v>
@@ -20577,13 +20577,13 @@
         <v>3</v>
       </c>
       <c r="K398">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L398">
         <v>2</v>
       </c>
       <c r="M398">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N398">
         <v>1</v>
@@ -20630,7 +20630,7 @@
         <v>1</v>
       </c>
       <c r="M399">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N399">
         <v>1</v>
@@ -20671,16 +20671,16 @@
         <v>3</v>
       </c>
       <c r="K400">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L400">
         <v>3</v>
       </c>
       <c r="M400">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N400">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O400">
         <v>6</v>
@@ -20762,7 +20762,7 @@
         <v>4</v>
       </c>
       <c r="J402">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K402">
         <v>5</v>

</xml_diff>